<commit_message>
minor adjustments for fresh print
</commit_message>
<xml_diff>
--- a/Master1.0.xlsx
+++ b/Master1.0.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kage\Documents\GitHub\Sculpt\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ntk\Documents\GitHub\Sculpt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AC2C0EC-688D-4CD3-B61B-578A631B7889}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{021DC251-7457-4539-BD0E-176CE36AEA0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet3" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="960" uniqueCount="576">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="960" uniqueCount="577">
   <si>
     <t>Name</t>
   </si>
@@ -2475,9 +2475,6 @@
 &lt;br&gt;&lt;b&gt;Extract energy:&lt;/b&gt; Refresh 1 chargeT.</t>
   </si>
   <si>
-    <t>Whenever you inflict a status effect, you may set that creature's composure to 1.</t>
-  </si>
-  <si>
     <t>When you make an attack, you may move 2 tiles before attacking.</t>
   </si>
   <si>
@@ -2545,9 +2542,81 @@
     <t>&lt;b&gt;Fire&lt;/b&gt; and &lt;b&gt;Burning&lt;/b&gt; give you temporary composure instead of dealing damage.</t>
   </si>
   <si>
+    <t>&lt;b&gt;Snigger:&lt;/b&gt; WeirdT or &lt;b&gt;Exhasusted&lt;/b&gt;</t>
+  </si>
+  <si>
+    <t>&lt;b&gt;Detonate: Exhaust&lt;/b&gt;</t>
+  </si>
+  <si>
+    <t>&lt;b&gt;Snap:&lt;/b&gt; 3 AP + &lt;b&gt;Exhaust&lt;/b&gt;</t>
+  </si>
+  <si>
+    <t>Whenever a being leaves your attack range, you may spend jazzT to make an attack with any limb against them. If the attack would cost 3 or more AP, &lt;b&gt;Exhaust&lt;/b&gt;.</t>
+  </si>
+  <si>
+    <t>You may clear a status effect (except &lt;b&gt;Exhausted&lt;/b&gt;) to refresh a token of your choice.</t>
+  </si>
+  <si>
+    <t>When you would take a status effect (except &lt;b&gt;Exhausted&lt;/b&gt;), ignore it instead.</t>
+  </si>
+  <si>
+    <t>Shovelling Talons</t>
+  </si>
+  <si>
+    <t>&lt;b&gt;Bloom:&lt;/b&gt;  WeirdT</t>
+  </si>
+  <si>
+    <t>Competely ignore damage from falling.</t>
+  </si>
+  <si>
+    <t>&lt;b&gt;Smear:&lt;/b&gt; 2 AP + weirdTweirdT</t>
+  </si>
+  <si>
+    <t>Engraved Slab</t>
+  </si>
+  <si>
+    <t>&lt;b&gt;Read the Runes:&lt;/b weirdT</t>
+  </si>
+  <si>
+    <t>Target being has half speed until the start of you next turn. (Each hex costs 2 move points)</t>
+  </si>
+  <si>
+    <t>&lt;B&gt;Slam:&lt;/b&gt; 4 AP</t>
+  </si>
+  <si>
+    <t>Storm Conduit</t>
+  </si>
+  <si>
+    <t>&lt;b&gt;Channel Storm:&lt;/b&gt; 2AP + weirdT</t>
+  </si>
+  <si>
+    <t>Create a 1 hex storm cloud at target empty hex.</t>
+  </si>
+  <si>
+    <t>&lt;b&gt;&lt;i&gt;Growing Storm&lt;/i&gt;&lt;/b&gt;</t>
+  </si>
+  <si>
+    <t>At the start of your turn, each storm cloud grows by one hex in all direction</t>
+  </si>
+  <si>
+    <t>&lt;B&gt;&lt;i&gt;Electrified&lt;/b&gt;&lt;/i&gt;</t>
+  </si>
+  <si>
+    <t>Whenever you spend weirdT, all beings underneath a storm cloud take 4 damage. This damage cannot be reduced.</t>
+  </si>
+  <si>
+    <t>Your second attack each turn costs 1 less AP.</t>
+  </si>
+  <si>
+    <t>&lt;b&gt;&lt;i&gt;Creative Duelist&lt;/i&gt;&lt;/b&gt;</t>
+  </si>
+  <si>
+    <t>Whenever you inflict a status effect, you may set that creatures composure to 1.</t>
+  </si>
+  <si>
     <r>
-      <t xml:space="preserve">&lt;b&gt;Increase damage taken by 1.&lt;/b&gt;
-&lt;br&gt;-1 </t>
+      <t xml:space="preserve">Reduce damage taken by 1.
+&lt;br&gt;- 1 </t>
     </r>
     <r>
       <rPr>
@@ -2570,73 +2639,29 @@
     </r>
   </si>
   <si>
-    <t>&lt;b&gt;Snigger:&lt;/b&gt; WeirdT or &lt;b&gt;Exhasusted&lt;/b&gt;</t>
-  </si>
-  <si>
-    <t>&lt;b&gt;Detonate: Exhaust&lt;/b&gt;</t>
-  </si>
-  <si>
-    <t>&lt;b&gt;Snap:&lt;/b&gt; 3 AP + &lt;b&gt;Exhaust&lt;/b&gt;</t>
-  </si>
-  <si>
-    <t>Whenever a being leaves your attack range, you may spend jazzT to make an attack with any limb against them. If the attack would cost 3 or more AP, &lt;b&gt;Exhaust&lt;/b&gt;.</t>
-  </si>
-  <si>
-    <t>You may clear a status effect (except &lt;b&gt;Exhausted&lt;/b&gt;) to refresh a token of your choice.</t>
-  </si>
-  <si>
-    <t>When you would take a status effect (except &lt;b&gt;Exhausted&lt;/b&gt;), ignore it instead.</t>
-  </si>
-  <si>
-    <t>Shovelling Talons</t>
-  </si>
-  <si>
-    <t>&lt;b&gt;Bloom:&lt;/b&gt;  WeirdT</t>
-  </si>
-  <si>
-    <t>Competely ignore damage from falling.</t>
-  </si>
-  <si>
-    <t>&lt;b&gt;Smear:&lt;/b&gt; 2 AP + weirdTweirdT</t>
-  </si>
-  <si>
-    <t>Engraved Slab</t>
-  </si>
-  <si>
-    <t>&lt;b&gt;Read the Runes:&lt;/b weirdT</t>
-  </si>
-  <si>
-    <t>Target being has half speed until the start of you next turn. (Each hex costs 2 move points)</t>
-  </si>
-  <si>
-    <t>&lt;B&gt;Slam:&lt;/b&gt; 4 AP</t>
-  </si>
-  <si>
-    <t>Storm Conduit</t>
-  </si>
-  <si>
-    <t>&lt;b&gt;Channel Storm:&lt;/b&gt; 2AP + weirdT</t>
-  </si>
-  <si>
-    <t>Create a 1 hex storm cloud at target empty hex.</t>
-  </si>
-  <si>
-    <t>&lt;b&gt;&lt;i&gt;Growing Storm&lt;/i&gt;&lt;/b&gt;</t>
-  </si>
-  <si>
-    <t>At the start of your turn, each storm cloud grows by one hex in all direction</t>
-  </si>
-  <si>
-    <t>&lt;B&gt;&lt;i&gt;Electrified&lt;/b&gt;&lt;/i&gt;</t>
-  </si>
-  <si>
-    <t>Whenever you spend weirdT, all beings underneath a storm cloud take 4 damage. This damage cannot be reduced.</t>
-  </si>
-  <si>
-    <t>Your second attack each turn costs 1 less AP.</t>
-  </si>
-  <si>
-    <t>&lt;b&gt;&lt;i&gt;Creative Duelist&lt;/i&gt;&lt;/b&gt;</t>
+    <r>
+      <t xml:space="preserve">&lt;b&gt;Increase damage taken by 1.&lt;/b&gt;
+&lt;br&gt;- 1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t>Movement Speed</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>.</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -3351,33 +3376,33 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AG199"/>
-  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
-    <col min="3" max="3" width="17.140625" customWidth="1"/>
-    <col min="4" max="4" width="1.42578125" customWidth="1"/>
-    <col min="5" max="5" width="4.28515625" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="3" max="3" width="17.109375" customWidth="1"/>
+    <col min="4" max="4" width="1.44140625" customWidth="1"/>
+    <col min="5" max="5" width="4.33203125" customWidth="1"/>
+    <col min="6" max="6" width="8.33203125" customWidth="1"/>
     <col min="7" max="7" width="33" customWidth="1"/>
-    <col min="8" max="8" width="42.42578125" customWidth="1"/>
-    <col min="9" max="9" width="1.42578125" customWidth="1"/>
-    <col min="10" max="10" width="6.85546875" customWidth="1"/>
-    <col min="11" max="11" width="14.85546875" customWidth="1"/>
-    <col min="12" max="12" width="31.7109375" customWidth="1"/>
-    <col min="13" max="13" width="37.85546875" style="24" customWidth="1"/>
-    <col min="14" max="14" width="1.42578125" customWidth="1"/>
-    <col min="15" max="15" width="6.5703125" customWidth="1"/>
-    <col min="16" max="16" width="8.42578125" customWidth="1"/>
-    <col min="17" max="17" width="25.5703125" customWidth="1"/>
-    <col min="18" max="18" width="35.140625" customWidth="1"/>
-    <col min="19" max="19" width="1.42578125" customWidth="1"/>
+    <col min="8" max="8" width="42.44140625" customWidth="1"/>
+    <col min="9" max="9" width="1.44140625" customWidth="1"/>
+    <col min="10" max="10" width="6.88671875" customWidth="1"/>
+    <col min="11" max="11" width="14.88671875" customWidth="1"/>
+    <col min="12" max="12" width="31.6640625" customWidth="1"/>
+    <col min="13" max="13" width="37.88671875" style="24" customWidth="1"/>
+    <col min="14" max="14" width="1.44140625" customWidth="1"/>
+    <col min="15" max="15" width="6.5546875" customWidth="1"/>
+    <col min="16" max="16" width="8.44140625" customWidth="1"/>
+    <col min="17" max="17" width="25.5546875" customWidth="1"/>
+    <col min="18" max="18" width="35.109375" customWidth="1"/>
+    <col min="19" max="19" width="1.44140625" customWidth="1"/>
     <col min="20" max="20" width="10" customWidth="1"/>
     <col min="21" max="21" width="38" customWidth="1"/>
-    <col min="24" max="31" width="10.5703125" customWidth="1"/>
+    <col min="24" max="31" width="10.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:33" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3478,7 +3503,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>29</v>
       </c>
@@ -3510,7 +3535,7 @@
         <v>34</v>
       </c>
       <c r="M2" s="6" t="s">
-        <v>537</v>
+        <v>574</v>
       </c>
       <c r="N2" s="21"/>
       <c r="O2" s="6"/>
@@ -3570,7 +3595,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="3" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>35</v>
       </c>
@@ -3606,7 +3631,7 @@
       </c>
       <c r="N3" s="21"/>
       <c r="O3" s="6">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="P3" s="8" t="s">
         <v>31</v>
@@ -3649,18 +3674,18 @@
       </c>
       <c r="AE3" s="6">
         <f>Table3[[#This Row],[E3Y]]+X$2</f>
-        <v>6.04</v>
+        <v>5.6</v>
       </c>
       <c r="AF3" s="6">
         <f>Table3[[#This Row],[E3TY]]+W$2</f>
-        <v>5.93</v>
+        <v>5.4899999999999993</v>
       </c>
       <c r="AG3" s="8">
         <f>T$2+U$2*(Table3[[#This Row],[Effect 3 Y]]-1)+2*V$2</f>
-        <v>6.64</v>
-      </c>
-    </row>
-    <row r="4" spans="1:33" ht="60" x14ac:dyDescent="0.25">
+        <v>6.1999999999999993</v>
+      </c>
+    </row>
+    <row r="4" spans="1:33" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>41</v>
       </c>
@@ -3746,7 +3771,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="5" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>47</v>
       </c>
@@ -3832,7 +3857,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="6" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>53</v>
       </c>
@@ -3908,9 +3933,9 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="7" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="26" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>30</v>
@@ -3926,10 +3951,10 @@
         <v>314</v>
       </c>
       <c r="G7" s="9" t="s">
+        <v>546</v>
+      </c>
+      <c r="H7" s="8" t="s">
         <v>547</v>
-      </c>
-      <c r="H7" s="8" t="s">
-        <v>548</v>
       </c>
       <c r="I7" s="7"/>
       <c r="J7" s="6">
@@ -3939,10 +3964,10 @@
         <v>31</v>
       </c>
       <c r="L7" s="8" t="s">
+        <v>548</v>
+      </c>
+      <c r="M7" s="6" t="s">
         <v>549</v>
-      </c>
-      <c r="M7" s="6" t="s">
-        <v>550</v>
       </c>
       <c r="N7" s="21"/>
       <c r="O7" s="6"/>
@@ -3992,7 +4017,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="8" spans="1:33" ht="75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:33" ht="72" x14ac:dyDescent="0.3">
       <c r="A8" s="26" t="s">
         <v>56</v>
       </c>
@@ -4074,7 +4099,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="9" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>61</v>
       </c>
@@ -4093,7 +4118,7 @@
         <v>62</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>552</v>
+        <v>576</v>
       </c>
       <c r="I9" s="7"/>
       <c r="J9" s="6">
@@ -4119,7 +4144,7 @@
         <v>65</v>
       </c>
       <c r="R9" s="6" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="S9" s="7"/>
       <c r="T9" s="6"/>
@@ -4164,7 +4189,7 @@
         <v>6.64</v>
       </c>
     </row>
-    <row r="10" spans="1:33" ht="60" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:33" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>66</v>
       </c>
@@ -4246,7 +4271,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="11" spans="1:33" ht="90" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:33" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>71</v>
       </c>
@@ -4267,7 +4292,7 @@
         <v>73</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>74</v>
+        <v>575</v>
       </c>
       <c r="I11" s="7"/>
       <c r="J11" s="6">
@@ -4330,7 +4355,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="12" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>77</v>
       </c>
@@ -4368,7 +4393,7 @@
       </c>
       <c r="N12" s="21"/>
       <c r="O12" s="6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="P12" s="8" t="s">
         <v>44</v>
@@ -4411,18 +4436,18 @@
       </c>
       <c r="AE12" s="6">
         <f>Table3[[#This Row],[E3Y]]+X$2</f>
-        <v>5.16</v>
+        <v>4.72</v>
       </c>
       <c r="AF12" s="6">
         <f>Table3[[#This Row],[E3TY]]+W$2</f>
-        <v>5.05</v>
+        <v>4.6099999999999994</v>
       </c>
       <c r="AG12" s="8">
         <f>T$2+U$2*(Table3[[#This Row],[Effect 3 Y]]-1)+2*V$2</f>
-        <v>5.76</v>
-      </c>
-    </row>
-    <row r="13" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+        <v>5.3199999999999994</v>
+      </c>
+    </row>
+    <row r="13" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>83</v>
       </c>
@@ -4445,7 +4470,7 @@
       </c>
       <c r="I13" s="7"/>
       <c r="J13" s="6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K13" s="8" t="s">
         <v>31</v>
@@ -4481,15 +4506,15 @@
       </c>
       <c r="AB13" s="6">
         <f>Table3[[#This Row],[E2Y]]+X$2</f>
-        <v>4.8600000000000003</v>
+        <v>4.42</v>
       </c>
       <c r="AC13" s="6">
         <f>Table3[[#This Row],[E2TY]]+W$2</f>
-        <v>4.75</v>
+        <v>4.3099999999999996</v>
       </c>
       <c r="AD13" s="6">
         <f>T$2+U$2*(Table3[[#This Row],[Effect 2 Y]]-1)+V$2</f>
-        <v>5.46</v>
+        <v>5.0199999999999996</v>
       </c>
       <c r="AE13" s="6">
         <f>Table3[[#This Row],[E3Y]]+X$2</f>
@@ -4504,7 +4529,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="14" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>87</v>
       </c>
@@ -4594,7 +4619,7 @@
         <v>6.64</v>
       </c>
     </row>
-    <row r="15" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>94</v>
       </c>
@@ -4686,7 +4711,7 @@
         <v>6.1999999999999993</v>
       </c>
     </row>
-    <row r="16" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>101</v>
       </c>
@@ -4764,7 +4789,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="17" spans="1:33" ht="60" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:33" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>103</v>
       </c>
@@ -4856,7 +4881,7 @@
         <v>7.08</v>
       </c>
     </row>
-    <row r="18" spans="1:33" ht="60" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>110</v>
       </c>
@@ -4875,7 +4900,7 @@
         <v>111</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="I18" s="7"/>
       <c r="J18" s="6">
@@ -4946,7 +4971,7 @@
         <v>5.76</v>
       </c>
     </row>
-    <row r="19" spans="1:33" ht="60" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:33" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
         <v>116</v>
       </c>
@@ -5028,7 +5053,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="20" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>121</v>
       </c>
@@ -5110,7 +5135,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="21" spans="1:33" ht="135" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:33" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>126</v>
       </c>
@@ -5194,7 +5219,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="22" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>131</v>
       </c>
@@ -5284,7 +5309,7 @@
         <v>5.76</v>
       </c>
     </row>
-    <row r="23" spans="1:33" ht="60" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:33" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
         <v>138</v>
       </c>
@@ -5331,7 +5356,7 @@
         <v>144</v>
       </c>
       <c r="R23" s="6" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="S23" s="7"/>
       <c r="T23" s="6"/>
@@ -5376,7 +5401,7 @@
         <v>6.1999999999999993</v>
       </c>
     </row>
-    <row r="24" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>145</v>
       </c>
@@ -5468,7 +5493,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="25" spans="1:33" ht="60" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:33" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
         <v>150</v>
       </c>
@@ -5550,7 +5575,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="26" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
         <v>154</v>
       </c>
@@ -5571,7 +5596,7 @@
         <v>155</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="I26" s="7"/>
       <c r="J26" s="6">
@@ -5642,7 +5667,7 @@
         <v>7.08</v>
       </c>
     </row>
-    <row r="27" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
         <v>160</v>
       </c>
@@ -5661,7 +5686,7 @@
         <v>161</v>
       </c>
       <c r="H27" s="8" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="I27" s="7"/>
       <c r="J27" s="6">
@@ -5687,7 +5712,7 @@
         <v>164</v>
       </c>
       <c r="R27" s="10" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="S27" s="7"/>
       <c r="T27" s="6"/>
@@ -5732,7 +5757,7 @@
         <v>6.64</v>
       </c>
     </row>
-    <row r="28" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>165</v>
       </c>
@@ -5814,7 +5839,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="29" spans="1:33" ht="60" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
         <v>170</v>
       </c>
@@ -5888,7 +5913,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="30" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
         <v>174</v>
       </c>
@@ -5907,7 +5932,7 @@
         <v>175</v>
       </c>
       <c r="H30" s="8" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="I30" s="7"/>
       <c r="J30" s="6">
@@ -5917,7 +5942,7 @@
         <v>31</v>
       </c>
       <c r="L30" s="6" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="M30" s="6" t="s">
         <v>176</v>
@@ -5970,7 +5995,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="31" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>177</v>
       </c>
@@ -5989,7 +6014,7 @@
         <v>178</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="I31" s="14"/>
       <c r="J31" s="6"/>
@@ -6044,7 +6069,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="32" spans="1:33" ht="75" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:33" ht="72" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
         <v>179</v>
       </c>
@@ -6118,7 +6143,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="33" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
         <v>182</v>
       </c>
@@ -6192,7 +6217,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="34" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
         <v>184</v>
       </c>
@@ -6266,7 +6291,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="35" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
         <v>186</v>
       </c>
@@ -6340,7 +6365,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="36" spans="1:33" ht="75" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:33" ht="72" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
         <v>190</v>
       </c>
@@ -6414,7 +6439,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="37" spans="1:33" ht="75" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:33" ht="72" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
         <v>192</v>
       </c>
@@ -6437,7 +6462,7 @@
       </c>
       <c r="I37" s="7"/>
       <c r="J37" s="6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K37" s="8" t="s">
         <v>31</v>
@@ -6473,15 +6498,15 @@
       </c>
       <c r="AB37" s="6">
         <f>Table3[[#This Row],[E2Y]]+X$2</f>
-        <v>4.8600000000000003</v>
+        <v>4.42</v>
       </c>
       <c r="AC37" s="6">
         <f>Table3[[#This Row],[E2TY]]+W$2</f>
-        <v>4.75</v>
+        <v>4.3099999999999996</v>
       </c>
       <c r="AD37" s="6">
         <f>T$2+U$2*(Table3[[#This Row],[Effect 2 Y]]-1)+V$2</f>
-        <v>5.46</v>
+        <v>5.0199999999999996</v>
       </c>
       <c r="AE37" s="6">
         <f>Table3[[#This Row],[E3Y]]+X$2</f>
@@ -6496,7 +6521,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="38" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
         <v>197</v>
       </c>
@@ -6515,7 +6540,7 @@
         <v>180</v>
       </c>
       <c r="H38" s="8" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="I38" s="7"/>
       <c r="J38" s="6"/>
@@ -6570,7 +6595,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="39" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A39" s="4" t="s">
         <v>198</v>
       </c>
@@ -6644,7 +6669,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="40" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A40" s="4" t="s">
         <v>200</v>
       </c>
@@ -6665,7 +6690,7 @@
         <v>202</v>
       </c>
       <c r="H40" s="8" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="I40" s="7"/>
       <c r="J40" s="6"/>
@@ -6720,7 +6745,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="41" spans="1:33" ht="60" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A41" s="4" t="s">
         <v>203</v>
       </c>
@@ -6802,7 +6827,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="42" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
         <v>208</v>
       </c>
@@ -6876,7 +6901,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="43" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A43" s="4" t="s">
         <v>210</v>
       </c>
@@ -6950,7 +6975,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="44" spans="1:33" ht="90" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:33" ht="72" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
         <v>212</v>
       </c>
@@ -6973,7 +6998,7 @@
       </c>
       <c r="I44" s="7"/>
       <c r="J44" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K44" s="8" t="s">
         <v>44</v>
@@ -6986,13 +7011,13 @@
       </c>
       <c r="N44" s="21"/>
       <c r="O44" s="6">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="P44" s="6" t="s">
         <v>44</v>
       </c>
       <c r="Q44" s="8" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="R44" s="6" t="s">
         <v>217</v>
@@ -7017,30 +7042,30 @@
       </c>
       <c r="AB44" s="6">
         <f>Table3[[#This Row],[E2Y]]+X$2</f>
-        <v>4.42</v>
+        <v>3.98</v>
       </c>
       <c r="AC44" s="6">
         <f>Table3[[#This Row],[E2TY]]+W$2</f>
-        <v>4.3099999999999996</v>
+        <v>3.87</v>
       </c>
       <c r="AD44" s="6">
         <f>T$2+U$2*(Table3[[#This Row],[Effect 2 Y]]-1)+V$2</f>
-        <v>5.0199999999999996</v>
+        <v>4.58</v>
       </c>
       <c r="AE44" s="6">
         <f>Table3[[#This Row],[E3Y]]+X$2</f>
-        <v>6.48</v>
+        <v>6.04</v>
       </c>
       <c r="AF44" s="6">
         <f>Table3[[#This Row],[E3TY]]+W$2</f>
-        <v>6.37</v>
+        <v>5.93</v>
       </c>
       <c r="AG44" s="8">
         <f>T$2+U$2*(Table3[[#This Row],[Effect 3 Y]]-1)+2*V$2</f>
-        <v>7.08</v>
-      </c>
-    </row>
-    <row r="45" spans="1:33" ht="60" x14ac:dyDescent="0.25">
+        <v>6.64</v>
+      </c>
+    </row>
+    <row r="45" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A45" s="4" t="s">
         <v>218</v>
       </c>
@@ -7122,7 +7147,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="46" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A46" s="4" t="s">
         <v>223</v>
       </c>
@@ -7198,7 +7223,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="47" spans="1:33" ht="60" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A47" s="4" t="s">
         <v>227</v>
       </c>
@@ -7221,7 +7246,7 @@
       </c>
       <c r="I47" s="7"/>
       <c r="J47" s="6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K47" s="8" t="s">
         <v>31</v>
@@ -7257,15 +7282,15 @@
       </c>
       <c r="AB47" s="6">
         <f>Table3[[#This Row],[E2Y]]+X$2</f>
-        <v>4.8600000000000003</v>
+        <v>4.42</v>
       </c>
       <c r="AC47" s="6">
         <f>Table3[[#This Row],[E2TY]]+W$2</f>
-        <v>4.75</v>
+        <v>4.3099999999999996</v>
       </c>
       <c r="AD47" s="6">
         <f>T$2+U$2*(Table3[[#This Row],[Effect 2 Y]]-1)+V$2</f>
-        <v>5.46</v>
+        <v>5.0199999999999996</v>
       </c>
       <c r="AE47" s="6">
         <f>Table3[[#This Row],[E3Y]]+X$2</f>
@@ -7280,7 +7305,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="48" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A48" s="4" t="s">
         <v>232</v>
       </c>
@@ -7354,7 +7379,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="49" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A49" s="4" t="s">
         <v>234</v>
       </c>
@@ -7436,7 +7461,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="50" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A50" s="4" t="s">
         <v>237</v>
       </c>
@@ -7510,7 +7535,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="51" spans="1:33" ht="75" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:33" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A51" s="4" t="s">
         <v>240</v>
       </c>
@@ -7592,7 +7617,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="52" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A52" s="4" t="s">
         <v>245</v>
       </c>
@@ -7666,7 +7691,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="53" spans="1:33" ht="90" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:33" ht="72" x14ac:dyDescent="0.3">
       <c r="A53" s="4" t="s">
         <v>248</v>
       </c>
@@ -7740,7 +7765,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="54" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A54" s="4" t="s">
         <v>251</v>
       </c>
@@ -7814,7 +7839,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="55" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A55" s="4" t="s">
         <v>254</v>
       </c>
@@ -7896,7 +7921,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="56" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A56" s="4" t="s">
         <v>259</v>
       </c>
@@ -7970,7 +7995,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="57" spans="1:33" ht="60" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A57" s="4" t="s">
         <v>260</v>
       </c>
@@ -8052,7 +8077,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="58" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A58" s="4" t="s">
         <v>265</v>
       </c>
@@ -8134,7 +8159,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="59" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A59" s="4" t="s">
         <v>270</v>
       </c>
@@ -8216,7 +8241,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="60" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A60" s="4" t="s">
         <v>275</v>
       </c>
@@ -8290,7 +8315,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="61" spans="1:33" ht="75" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:33" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A61" s="4" t="s">
         <v>277</v>
       </c>
@@ -8372,7 +8397,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="62" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A62" s="4" t="s">
         <v>282</v>
       </c>
@@ -8446,7 +8471,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="63" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A63" s="4" t="s">
         <v>284</v>
       </c>
@@ -8520,7 +8545,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="64" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A64" s="4" t="s">
         <v>287</v>
       </c>
@@ -8539,7 +8564,7 @@
         <v>288</v>
       </c>
       <c r="H64" s="8" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="I64" s="7"/>
       <c r="J64" s="6"/>
@@ -8594,7 +8619,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="65" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A65" s="4" t="s">
         <v>289</v>
       </c>
@@ -8676,7 +8701,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="66" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A66" s="4" t="s">
         <v>294</v>
       </c>
@@ -8750,7 +8775,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="67" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A67" s="4" t="s">
         <v>296</v>
       </c>
@@ -8766,14 +8791,14 @@
         <v>187</v>
       </c>
       <c r="G67" s="8" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="H67" s="8" t="s">
         <v>297</v>
       </c>
       <c r="I67" s="7"/>
       <c r="J67" s="6">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K67" s="6" t="s">
         <v>31</v>
@@ -8809,15 +8834,15 @@
       </c>
       <c r="AB67" s="6">
         <f>Table3[[#This Row],[E2Y]]+X$2</f>
-        <v>5.3</v>
+        <v>4.8600000000000003</v>
       </c>
       <c r="AC67" s="6">
         <f>Table3[[#This Row],[E2TY]]+W$2</f>
-        <v>5.1899999999999995</v>
+        <v>4.75</v>
       </c>
       <c r="AD67" s="6">
         <f>T$2+U$2*(Table3[[#This Row],[Effect 2 Y]]-1)+V$2</f>
-        <v>5.8999999999999995</v>
+        <v>5.46</v>
       </c>
       <c r="AE67" s="6">
         <f>Table3[[#This Row],[E3Y]]+X$2</f>
@@ -8832,7 +8857,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="68" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A68" s="4" t="s">
         <v>300</v>
       </c>
@@ -8906,7 +8931,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="69" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A69" s="4" t="s">
         <v>303</v>
       </c>
@@ -8988,7 +9013,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="70" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A70" s="4" t="s">
         <v>307</v>
       </c>
@@ -9062,7 +9087,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="71" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A71" s="4" t="s">
         <v>310</v>
       </c>
@@ -9152,7 +9177,7 @@
         <v>7.3</v>
       </c>
     </row>
-    <row r="72" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A72" s="4" t="s">
         <v>320</v>
       </c>
@@ -9236,7 +9261,7 @@
         <v>5.3199999999999994</v>
       </c>
     </row>
-    <row r="73" spans="1:33" ht="60" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A73" s="4" t="s">
         <v>324</v>
       </c>
@@ -9318,7 +9343,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="74" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A74" s="4" t="s">
         <v>329</v>
       </c>
@@ -9402,7 +9427,7 @@
         <v>5.3199999999999994</v>
       </c>
     </row>
-    <row r="75" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A75" s="4" t="s">
         <v>334</v>
       </c>
@@ -9484,7 +9509,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="76" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A76" s="4" t="s">
         <v>339</v>
       </c>
@@ -9566,7 +9591,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="77" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A77" s="4" t="s">
         <v>344</v>
       </c>
@@ -9648,7 +9673,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="78" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A78" s="4" t="s">
         <v>347</v>
       </c>
@@ -9730,7 +9755,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="79" spans="1:33" ht="75" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:33" ht="72" x14ac:dyDescent="0.3">
       <c r="A79" s="4" t="s">
         <v>352</v>
       </c>
@@ -9812,7 +9837,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="80" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A80" s="4" t="s">
         <v>356</v>
       </c>
@@ -9894,7 +9919,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="81" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A81" s="4" t="s">
         <v>361</v>
       </c>
@@ -9923,7 +9948,7 @@
         <v>44</v>
       </c>
       <c r="L81" s="6" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="M81" s="6" t="s">
         <v>364</v>
@@ -9984,7 +10009,7 @@
         <v>7.3</v>
       </c>
     </row>
-    <row r="82" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A82" s="4" t="s">
         <v>366</v>
       </c>
@@ -10074,9 +10099,9 @@
         <v>7.3</v>
       </c>
     </row>
-    <row r="83" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A83" s="4" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="B83" s="15" t="s">
         <v>311</v>
@@ -10090,10 +10115,10 @@
         <v>44</v>
       </c>
       <c r="G83" s="8" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="H83" s="8" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="I83" s="7"/>
       <c r="J83" s="6">
@@ -10103,7 +10128,7 @@
         <v>314</v>
       </c>
       <c r="L83" s="6" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="M83" s="6" t="s">
         <v>379</v>
@@ -10156,7 +10181,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="84" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A84" s="4" t="s">
         <v>371</v>
       </c>
@@ -10230,7 +10255,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="85" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A85" s="4" t="s">
         <v>374</v>
       </c>
@@ -10261,7 +10286,7 @@
         <v>187</v>
       </c>
       <c r="L85" s="6" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="M85" s="6" t="s">
         <v>377</v>
@@ -10314,7 +10339,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="86" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A86" s="4" t="s">
         <v>378</v>
       </c>
@@ -10396,7 +10421,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="87" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A87" s="4" t="s">
         <v>381</v>
       </c>
@@ -10486,7 +10511,7 @@
         <v>7.3</v>
       </c>
     </row>
-    <row r="88" spans="1:33" ht="60" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A88" s="4" t="s">
         <v>386</v>
       </c>
@@ -10560,7 +10585,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="89" spans="1:33" ht="75" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:33" ht="72" x14ac:dyDescent="0.3">
       <c r="A89" s="4" t="s">
         <v>389</v>
       </c>
@@ -10642,7 +10667,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="90" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A90" s="4" t="s">
         <v>394</v>
       </c>
@@ -10724,7 +10749,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="91" spans="1:33" ht="75" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:33" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A91" s="4" t="s">
         <v>398</v>
       </c>
@@ -10806,7 +10831,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="92" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A92" s="4" t="s">
         <v>402</v>
       </c>
@@ -10835,10 +10860,10 @@
         <v>187</v>
       </c>
       <c r="L92" s="6" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="M92" s="6" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="N92" s="21"/>
       <c r="O92" s="6"/>
@@ -10888,7 +10913,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="93" spans="1:33" ht="75" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:33" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A93" s="4" t="s">
         <v>405</v>
       </c>
@@ -10972,7 +10997,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="94" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A94" s="4" t="s">
         <v>411</v>
       </c>
@@ -11054,7 +11079,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="95" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A95" s="4" t="s">
         <v>415</v>
       </c>
@@ -11077,7 +11102,7 @@
       </c>
       <c r="I95" s="7"/>
       <c r="J95" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K95" s="6" t="s">
         <v>31</v>
@@ -11113,15 +11138,15 @@
       </c>
       <c r="AB95" s="6">
         <f>Table3[[#This Row],[E2Y]]+X$2</f>
-        <v>4.42</v>
+        <v>3.98</v>
       </c>
       <c r="AC95" s="6">
         <f>Table3[[#This Row],[E2TY]]+W$2</f>
-        <v>4.3099999999999996</v>
+        <v>3.87</v>
       </c>
       <c r="AD95" s="6">
         <f>T$2+U$2*(Table3[[#This Row],[Effect 2 Y]]-1)+V$2</f>
-        <v>5.0199999999999996</v>
+        <v>4.58</v>
       </c>
       <c r="AE95" s="6">
         <f>Table3[[#This Row],[E3Y]]+X$2</f>
@@ -11136,7 +11161,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="96" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A96" s="4" t="s">
         <v>420</v>
       </c>
@@ -11218,7 +11243,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="97" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A97" s="4" t="s">
         <v>423</v>
       </c>
@@ -11300,7 +11325,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="98" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A98" s="4" t="s">
         <v>428</v>
       </c>
@@ -11336,7 +11361,7 @@
       </c>
       <c r="N98" s="21"/>
       <c r="O98" s="6">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="P98" s="6" t="s">
         <v>317</v>
@@ -11379,18 +11404,18 @@
       </c>
       <c r="AE98" s="6">
         <f>Table3[[#This Row],[E3Y]]+X$2</f>
-        <v>6.92</v>
+        <v>7.36</v>
       </c>
       <c r="AF98" s="6">
         <f>Table3[[#This Row],[E3TY]]+W$2</f>
-        <v>6.81</v>
+        <v>7.25</v>
       </c>
       <c r="AG98" s="8">
         <f>T$2+U$2*(Table3[[#This Row],[Effect 3 Y]]-1)+2*V$2</f>
-        <v>7.52</v>
-      </c>
-    </row>
-    <row r="99" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+        <v>7.96</v>
+      </c>
+    </row>
+    <row r="99" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A99" s="4" t="s">
         <v>433</v>
       </c>
@@ -11464,7 +11489,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="100" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A100" s="4" t="s">
         <v>436</v>
       </c>
@@ -11480,7 +11505,7 @@
         <v>314</v>
       </c>
       <c r="G100" s="8" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="H100" s="8" t="s">
         <v>437</v>
@@ -11538,7 +11563,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="101" spans="1:33" ht="75" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:33" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A101" s="4" t="s">
         <v>438</v>
       </c>
@@ -11628,7 +11653,7 @@
         <v>7.52</v>
       </c>
     </row>
-    <row r="102" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A102" s="4" t="s">
         <v>444</v>
       </c>
@@ -11710,7 +11735,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="103" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A103" s="4" t="s">
         <v>446</v>
       </c>
@@ -11784,7 +11809,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="104" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A104" s="4" t="s">
         <v>449</v>
       </c>
@@ -11866,7 +11891,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="105" spans="1:33" ht="60" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:33" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A105" s="4" t="s">
         <v>454</v>
       </c>
@@ -11950,7 +11975,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="106" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A106" s="4" t="s">
         <v>459</v>
       </c>
@@ -12034,9 +12059,9 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="107" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A107" s="4" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="B107" s="15" t="s">
         <v>311</v>
@@ -12124,7 +12149,7 @@
         <v>7.52</v>
       </c>
     </row>
-    <row r="108" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A108" s="4" t="s">
         <v>468</v>
       </c>
@@ -12206,7 +12231,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="109" spans="1:33" ht="60" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:33" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A109" s="4" t="s">
         <v>472</v>
       </c>
@@ -12290,7 +12315,7 @@
         <v>5.3199999999999994</v>
       </c>
     </row>
-    <row r="110" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A110" s="4" t="s">
         <v>477</v>
       </c>
@@ -12372,7 +12397,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="111" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A111" s="4" t="s">
         <v>481</v>
       </c>
@@ -12454,7 +12479,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="112" spans="1:33" ht="60" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:33" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A112" s="4" t="s">
         <v>484</v>
       </c>
@@ -12536,7 +12561,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="113" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A113" s="4" t="s">
         <v>488</v>
       </c>
@@ -12610,9 +12635,9 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="114" spans="1:33" ht="60" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A114" s="4" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="B114" s="15" t="s">
         <v>311</v>
@@ -12626,10 +12651,10 @@
         <v>44</v>
       </c>
       <c r="G114" s="8" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="H114" s="8" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="I114" s="7"/>
       <c r="J114" s="6">
@@ -12639,23 +12664,23 @@
         <v>31</v>
       </c>
       <c r="L114" s="6" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="M114" s="6" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="N114" s="21"/>
       <c r="O114" s="6">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P114" s="6" t="s">
         <v>31</v>
       </c>
       <c r="Q114" s="6" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="R114" s="6" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="S114" s="7"/>
       <c r="T114" s="6"/>
@@ -12689,18 +12714,18 @@
       </c>
       <c r="AE114" s="6">
         <f>Table3[[#This Row],[E3Y]]+X$2</f>
-        <v>5.6</v>
+        <v>6.04</v>
       </c>
       <c r="AF114" s="6">
         <f>Table3[[#This Row],[E3TY]]+W$2</f>
-        <v>5.4899999999999993</v>
+        <v>5.93</v>
       </c>
       <c r="AG114" s="8">
         <f>T$2+U$2*(Table3[[#This Row],[Effect 3 Y]]-1)+2*V$2</f>
-        <v>6.1999999999999993</v>
-      </c>
-    </row>
-    <row r="115" spans="1:33" ht="75" x14ac:dyDescent="0.25">
+        <v>6.64</v>
+      </c>
+    </row>
+    <row r="115" spans="1:33" ht="72" x14ac:dyDescent="0.3">
       <c r="A115" s="4" t="s">
         <v>491</v>
       </c>
@@ -12774,7 +12799,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="116" spans="1:33" ht="75" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:33" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A116" s="4" t="s">
         <v>494</v>
       </c>
@@ -12856,7 +12881,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="117" spans="1:33" ht="75" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:33" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A117" s="4" t="s">
         <v>499</v>
       </c>
@@ -12888,7 +12913,7 @@
         <v>501</v>
       </c>
       <c r="M117" s="8" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
       <c r="N117" s="21"/>
       <c r="O117" s="6"/>
@@ -12938,7 +12963,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="118" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A118" s="4" t="s">
         <v>502</v>
       </c>
@@ -13028,7 +13053,7 @@
         <v>7.52</v>
       </c>
     </row>
-    <row r="119" spans="1:33" ht="60" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:33" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A119" s="4" t="s">
         <v>508</v>
       </c>
@@ -13110,7 +13135,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="120" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A120" s="4" t="s">
         <v>512</v>
       </c>
@@ -13184,7 +13209,7 @@
         <v>3.12</v>
       </c>
     </row>
-    <row r="121" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A121" s="18"/>
       <c r="B121" s="18"/>
       <c r="C121" s="18"/>
@@ -13219,7 +13244,7 @@
       <c r="AF121" s="18"/>
       <c r="AG121" s="19"/>
     </row>
-    <row r="122" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A122" s="18"/>
       <c r="B122" s="18"/>
       <c r="C122" s="18"/>
@@ -13254,7 +13279,7 @@
       <c r="AF122" s="18"/>
       <c r="AG122" s="19"/>
     </row>
-    <row r="123" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A123" s="18"/>
       <c r="B123" s="18"/>
       <c r="C123" s="18"/>
@@ -13289,7 +13314,7 @@
       <c r="AF123" s="18"/>
       <c r="AG123" s="19"/>
     </row>
-    <row r="124" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A124" s="18"/>
       <c r="B124" s="18"/>
       <c r="C124" s="18"/>
@@ -13324,7 +13349,7 @@
       <c r="AF124" s="18"/>
       <c r="AG124" s="19"/>
     </row>
-    <row r="125" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A125" s="18"/>
       <c r="B125" s="18"/>
       <c r="C125" s="18"/>
@@ -13359,7 +13384,7 @@
       <c r="AF125" s="18"/>
       <c r="AG125" s="19"/>
     </row>
-    <row r="126" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A126" s="18"/>
       <c r="B126" s="18"/>
       <c r="C126" s="18"/>
@@ -13394,7 +13419,7 @@
       <c r="AF126" s="18"/>
       <c r="AG126" s="19"/>
     </row>
-    <row r="127" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A127" s="18"/>
       <c r="B127" s="18"/>
       <c r="C127" s="18"/>
@@ -13429,7 +13454,7 @@
       <c r="AF127" s="18"/>
       <c r="AG127" s="19"/>
     </row>
-    <row r="128" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A128" s="18"/>
       <c r="B128" s="18"/>
       <c r="C128" s="18"/>
@@ -13464,7 +13489,7 @@
       <c r="AF128" s="18"/>
       <c r="AG128" s="19"/>
     </row>
-    <row r="129" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A129" s="18"/>
       <c r="B129" s="18"/>
       <c r="C129" s="18"/>
@@ -13499,7 +13524,7 @@
       <c r="AF129" s="18"/>
       <c r="AG129" s="19"/>
     </row>
-    <row r="130" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A130" s="18"/>
       <c r="B130" s="18"/>
       <c r="C130" s="18"/>
@@ -13534,7 +13559,7 @@
       <c r="AF130" s="18"/>
       <c r="AG130" s="19"/>
     </row>
-    <row r="131" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A131" s="18"/>
       <c r="B131" s="18"/>
       <c r="C131" s="18"/>
@@ -13569,7 +13594,7 @@
       <c r="AF131" s="18"/>
       <c r="AG131" s="19"/>
     </row>
-    <row r="132" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A132" s="18"/>
       <c r="B132" s="18"/>
       <c r="C132" s="18"/>
@@ -13604,7 +13629,7 @@
       <c r="AF132" s="18"/>
       <c r="AG132" s="19"/>
     </row>
-    <row r="133" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A133" s="18"/>
       <c r="B133" s="18"/>
       <c r="C133" s="18"/>
@@ -13639,7 +13664,7 @@
       <c r="AF133" s="18"/>
       <c r="AG133" s="19"/>
     </row>
-    <row r="134" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A134" s="18"/>
       <c r="B134" s="18"/>
       <c r="C134" s="18"/>
@@ -13674,7 +13699,7 @@
       <c r="AF134" s="18"/>
       <c r="AG134" s="19"/>
     </row>
-    <row r="135" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A135" s="18"/>
       <c r="B135" s="18"/>
       <c r="C135" s="18"/>
@@ -13709,7 +13734,7 @@
       <c r="AF135" s="18"/>
       <c r="AG135" s="19"/>
     </row>
-    <row r="136" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A136" s="18"/>
       <c r="B136" s="18"/>
       <c r="C136" s="18"/>
@@ -13744,7 +13769,7 @@
       <c r="AF136" s="18"/>
       <c r="AG136" s="19"/>
     </row>
-    <row r="137" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A137" s="18"/>
       <c r="B137" s="18"/>
       <c r="C137" s="18"/>
@@ -13779,7 +13804,7 @@
       <c r="AF137" s="18"/>
       <c r="AG137" s="19"/>
     </row>
-    <row r="138" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A138" s="18"/>
       <c r="B138" s="18"/>
       <c r="C138" s="18"/>
@@ -13814,7 +13839,7 @@
       <c r="AF138" s="18"/>
       <c r="AG138" s="19"/>
     </row>
-    <row r="139" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A139" s="18"/>
       <c r="B139" s="18"/>
       <c r="C139" s="18"/>
@@ -13849,7 +13874,7 @@
       <c r="AF139" s="18"/>
       <c r="AG139" s="19"/>
     </row>
-    <row r="140" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A140" s="18"/>
       <c r="B140" s="18"/>
       <c r="C140" s="18"/>
@@ -13884,7 +13909,7 @@
       <c r="AF140" s="18"/>
       <c r="AG140" s="19"/>
     </row>
-    <row r="141" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A141" s="18"/>
       <c r="B141" s="18"/>
       <c r="C141" s="18"/>
@@ -13919,7 +13944,7 @@
       <c r="AF141" s="18"/>
       <c r="AG141" s="19"/>
     </row>
-    <row r="142" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A142" s="18"/>
       <c r="B142" s="18"/>
       <c r="C142" s="18"/>
@@ -13954,7 +13979,7 @@
       <c r="AF142" s="18"/>
       <c r="AG142" s="19"/>
     </row>
-    <row r="143" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A143" s="18"/>
       <c r="B143" s="18"/>
       <c r="C143" s="18"/>
@@ -13989,7 +14014,7 @@
       <c r="AF143" s="18"/>
       <c r="AG143" s="19"/>
     </row>
-    <row r="144" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A144" s="18"/>
       <c r="B144" s="18"/>
       <c r="C144" s="18"/>
@@ -14024,7 +14049,7 @@
       <c r="AF144" s="18"/>
       <c r="AG144" s="19"/>
     </row>
-    <row r="145" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A145" s="18"/>
       <c r="B145" s="18"/>
       <c r="C145" s="18"/>
@@ -14059,7 +14084,7 @@
       <c r="AF145" s="18"/>
       <c r="AG145" s="19"/>
     </row>
-    <row r="146" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A146" s="18"/>
       <c r="B146" s="18"/>
       <c r="C146" s="18"/>
@@ -14094,7 +14119,7 @@
       <c r="AF146" s="18"/>
       <c r="AG146" s="19"/>
     </row>
-    <row r="147" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A147" s="18"/>
       <c r="B147" s="18"/>
       <c r="C147" s="18"/>
@@ -14129,7 +14154,7 @@
       <c r="AF147" s="18"/>
       <c r="AG147" s="19"/>
     </row>
-    <row r="148" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A148" s="18"/>
       <c r="B148" s="18"/>
       <c r="C148" s="18"/>
@@ -14164,7 +14189,7 @@
       <c r="AF148" s="18"/>
       <c r="AG148" s="19"/>
     </row>
-    <row r="149" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A149" s="18"/>
       <c r="B149" s="18"/>
       <c r="C149" s="18"/>
@@ -14199,7 +14224,7 @@
       <c r="AF149" s="18"/>
       <c r="AG149" s="19"/>
     </row>
-    <row r="150" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A150" s="18"/>
       <c r="B150" s="18"/>
       <c r="C150" s="18"/>
@@ -14234,7 +14259,7 @@
       <c r="AF150" s="18"/>
       <c r="AG150" s="19"/>
     </row>
-    <row r="151" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A151" s="18"/>
       <c r="B151" s="18"/>
       <c r="C151" s="18"/>
@@ -14269,7 +14294,7 @@
       <c r="AF151" s="18"/>
       <c r="AG151" s="19"/>
     </row>
-    <row r="152" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A152" s="18"/>
       <c r="B152" s="18"/>
       <c r="C152" s="18"/>
@@ -14304,7 +14329,7 @@
       <c r="AF152" s="18"/>
       <c r="AG152" s="19"/>
     </row>
-    <row r="153" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A153" s="18"/>
       <c r="B153" s="18"/>
       <c r="C153" s="18"/>
@@ -14339,7 +14364,7 @@
       <c r="AF153" s="18"/>
       <c r="AG153" s="19"/>
     </row>
-    <row r="154" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A154" s="18"/>
       <c r="B154" s="18"/>
       <c r="C154" s="18"/>
@@ -14374,7 +14399,7 @@
       <c r="AF154" s="18"/>
       <c r="AG154" s="19"/>
     </row>
-    <row r="155" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A155" s="18"/>
       <c r="B155" s="18"/>
       <c r="C155" s="18"/>
@@ -14409,7 +14434,7 @@
       <c r="AF155" s="18"/>
       <c r="AG155" s="19"/>
     </row>
-    <row r="156" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A156" s="18"/>
       <c r="B156" s="18"/>
       <c r="C156" s="18"/>
@@ -14444,7 +14469,7 @@
       <c r="AF156" s="18"/>
       <c r="AG156" s="19"/>
     </row>
-    <row r="157" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A157" s="18"/>
       <c r="B157" s="18"/>
       <c r="C157" s="18"/>
@@ -14479,7 +14504,7 @@
       <c r="AF157" s="18"/>
       <c r="AG157" s="19"/>
     </row>
-    <row r="158" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A158" s="18"/>
       <c r="B158" s="18"/>
       <c r="C158" s="18"/>
@@ -14514,7 +14539,7 @@
       <c r="AF158" s="18"/>
       <c r="AG158" s="19"/>
     </row>
-    <row r="159" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A159" s="18"/>
       <c r="B159" s="18"/>
       <c r="C159" s="18"/>
@@ -14549,7 +14574,7 @@
       <c r="AF159" s="18"/>
       <c r="AG159" s="19"/>
     </row>
-    <row r="160" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A160" s="18"/>
       <c r="B160" s="18"/>
       <c r="C160" s="18"/>
@@ -14584,7 +14609,7 @@
       <c r="AF160" s="18"/>
       <c r="AG160" s="19"/>
     </row>
-    <row r="161" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A161" s="18"/>
       <c r="B161" s="18"/>
       <c r="C161" s="18"/>
@@ -14619,7 +14644,7 @@
       <c r="AF161" s="18"/>
       <c r="AG161" s="19"/>
     </row>
-    <row r="162" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A162" s="18"/>
       <c r="B162" s="18"/>
       <c r="C162" s="18"/>
@@ -14654,7 +14679,7 @@
       <c r="AF162" s="18"/>
       <c r="AG162" s="19"/>
     </row>
-    <row r="163" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A163" s="18"/>
       <c r="B163" s="18"/>
       <c r="C163" s="18"/>
@@ -14689,7 +14714,7 @@
       <c r="AF163" s="18"/>
       <c r="AG163" s="19"/>
     </row>
-    <row r="164" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A164" s="18"/>
       <c r="B164" s="18"/>
       <c r="C164" s="18"/>
@@ -14724,7 +14749,7 @@
       <c r="AF164" s="18"/>
       <c r="AG164" s="19"/>
     </row>
-    <row r="165" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A165" s="18"/>
       <c r="B165" s="18"/>
       <c r="C165" s="18"/>
@@ -14759,7 +14784,7 @@
       <c r="AF165" s="18"/>
       <c r="AG165" s="19"/>
     </row>
-    <row r="166" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A166" s="18"/>
       <c r="B166" s="18"/>
       <c r="C166" s="18"/>
@@ -14794,7 +14819,7 @@
       <c r="AF166" s="18"/>
       <c r="AG166" s="19"/>
     </row>
-    <row r="167" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A167" s="18"/>
       <c r="B167" s="18"/>
       <c r="C167" s="18"/>
@@ -14829,7 +14854,7 @@
       <c r="AF167" s="18"/>
       <c r="AG167" s="19"/>
     </row>
-    <row r="168" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A168" s="18"/>
       <c r="B168" s="18"/>
       <c r="C168" s="18"/>
@@ -14864,7 +14889,7 @@
       <c r="AF168" s="18"/>
       <c r="AG168" s="19"/>
     </row>
-    <row r="169" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A169" s="18"/>
       <c r="B169" s="18"/>
       <c r="C169" s="18"/>
@@ -14899,7 +14924,7 @@
       <c r="AF169" s="18"/>
       <c r="AG169" s="19"/>
     </row>
-    <row r="170" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A170" s="18"/>
       <c r="B170" s="18"/>
       <c r="C170" s="18"/>
@@ -14934,7 +14959,7 @@
       <c r="AF170" s="18"/>
       <c r="AG170" s="19"/>
     </row>
-    <row r="171" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A171" s="18"/>
       <c r="B171" s="18"/>
       <c r="C171" s="18"/>
@@ -14969,7 +14994,7 @@
       <c r="AF171" s="18"/>
       <c r="AG171" s="19"/>
     </row>
-    <row r="172" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A172" s="18"/>
       <c r="B172" s="18"/>
       <c r="C172" s="18"/>
@@ -15004,7 +15029,7 @@
       <c r="AF172" s="18"/>
       <c r="AG172" s="19"/>
     </row>
-    <row r="173" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A173" s="18"/>
       <c r="B173" s="18"/>
       <c r="C173" s="18"/>
@@ -15039,7 +15064,7 @@
       <c r="AF173" s="18"/>
       <c r="AG173" s="19"/>
     </row>
-    <row r="174" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A174" s="18"/>
       <c r="B174" s="18"/>
       <c r="C174" s="18"/>
@@ -15074,7 +15099,7 @@
       <c r="AF174" s="18"/>
       <c r="AG174" s="19"/>
     </row>
-    <row r="175" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A175" s="18"/>
       <c r="B175" s="18"/>
       <c r="C175" s="18"/>
@@ -15109,7 +15134,7 @@
       <c r="AF175" s="18"/>
       <c r="AG175" s="19"/>
     </row>
-    <row r="176" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A176" s="18"/>
       <c r="B176" s="18"/>
       <c r="C176" s="18"/>
@@ -15144,7 +15169,7 @@
       <c r="AF176" s="18"/>
       <c r="AG176" s="19"/>
     </row>
-    <row r="177" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A177" s="18"/>
       <c r="B177" s="18"/>
       <c r="C177" s="18"/>
@@ -15179,7 +15204,7 @@
       <c r="AF177" s="18"/>
       <c r="AG177" s="19"/>
     </row>
-    <row r="178" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A178" s="18"/>
       <c r="B178" s="18"/>
       <c r="C178" s="18"/>
@@ -15214,7 +15239,7 @@
       <c r="AF178" s="18"/>
       <c r="AG178" s="19"/>
     </row>
-    <row r="179" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A179" s="18"/>
       <c r="B179" s="18"/>
       <c r="C179" s="18"/>
@@ -15249,7 +15274,7 @@
       <c r="AF179" s="18"/>
       <c r="AG179" s="19"/>
     </row>
-    <row r="180" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A180" s="18"/>
       <c r="B180" s="18"/>
       <c r="C180" s="18"/>
@@ -15284,7 +15309,7 @@
       <c r="AF180" s="18"/>
       <c r="AG180" s="19"/>
     </row>
-    <row r="181" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A181" s="18"/>
       <c r="B181" s="18"/>
       <c r="C181" s="18"/>
@@ -15319,7 +15344,7 @@
       <c r="AF181" s="18"/>
       <c r="AG181" s="19"/>
     </row>
-    <row r="182" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A182" s="18"/>
       <c r="B182" s="18"/>
       <c r="C182" s="18"/>
@@ -15354,7 +15379,7 @@
       <c r="AF182" s="18"/>
       <c r="AG182" s="19"/>
     </row>
-    <row r="183" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A183" s="18"/>
       <c r="B183" s="18"/>
       <c r="C183" s="18"/>
@@ -15389,7 +15414,7 @@
       <c r="AF183" s="18"/>
       <c r="AG183" s="19"/>
     </row>
-    <row r="184" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A184" s="18"/>
       <c r="B184" s="18"/>
       <c r="C184" s="18"/>
@@ -15424,7 +15449,7 @@
       <c r="AF184" s="18"/>
       <c r="AG184" s="19"/>
     </row>
-    <row r="185" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A185" s="18"/>
       <c r="B185" s="18"/>
       <c r="C185" s="18"/>
@@ -15459,7 +15484,7 @@
       <c r="AF185" s="18"/>
       <c r="AG185" s="19"/>
     </row>
-    <row r="186" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A186" s="18"/>
       <c r="B186" s="18"/>
       <c r="C186" s="18"/>
@@ -15494,7 +15519,7 @@
       <c r="AF186" s="18"/>
       <c r="AG186" s="19"/>
     </row>
-    <row r="187" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A187" s="18"/>
       <c r="B187" s="18"/>
       <c r="C187" s="18"/>
@@ -15529,7 +15554,7 @@
       <c r="AF187" s="18"/>
       <c r="AG187" s="19"/>
     </row>
-    <row r="188" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A188" s="18"/>
       <c r="B188" s="18"/>
       <c r="C188" s="18"/>
@@ -15564,7 +15589,7 @@
       <c r="AF188" s="18"/>
       <c r="AG188" s="19"/>
     </row>
-    <row r="189" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A189" s="18"/>
       <c r="B189" s="18"/>
       <c r="C189" s="18"/>
@@ -15599,7 +15624,7 @@
       <c r="AF189" s="18"/>
       <c r="AG189" s="19"/>
     </row>
-    <row r="190" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A190" s="18"/>
       <c r="B190" s="18"/>
       <c r="C190" s="18"/>
@@ -15634,7 +15659,7 @@
       <c r="AF190" s="18"/>
       <c r="AG190" s="19"/>
     </row>
-    <row r="191" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A191" s="18"/>
       <c r="B191" s="18"/>
       <c r="C191" s="18"/>
@@ -15669,7 +15694,7 @@
       <c r="AF191" s="18"/>
       <c r="AG191" s="19"/>
     </row>
-    <row r="192" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A192" s="18"/>
       <c r="B192" s="18"/>
       <c r="C192" s="18"/>
@@ -15704,7 +15729,7 @@
       <c r="AF192" s="18"/>
       <c r="AG192" s="19"/>
     </row>
-    <row r="193" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A193" s="18"/>
       <c r="B193" s="18"/>
       <c r="C193" s="18"/>
@@ -15739,7 +15764,7 @@
       <c r="AF193" s="18"/>
       <c r="AG193" s="19"/>
     </row>
-    <row r="194" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A194" s="18"/>
       <c r="B194" s="18"/>
       <c r="C194" s="18"/>
@@ -15774,7 +15799,7 @@
       <c r="AF194" s="18"/>
       <c r="AG194" s="19"/>
     </row>
-    <row r="195" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A195" s="18"/>
       <c r="B195" s="18"/>
       <c r="C195" s="18"/>
@@ -15809,7 +15834,7 @@
       <c r="AF195" s="18"/>
       <c r="AG195" s="19"/>
     </row>
-    <row r="196" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A196" s="18"/>
       <c r="B196" s="18"/>
       <c r="C196" s="18"/>
@@ -15844,7 +15869,7 @@
       <c r="AF196" s="18"/>
       <c r="AG196" s="19"/>
     </row>
-    <row r="197" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A197" s="18"/>
       <c r="B197" s="18"/>
       <c r="C197" s="18"/>
@@ -15879,7 +15904,7 @@
       <c r="AF197" s="18"/>
       <c r="AG197" s="19"/>
     </row>
-    <row r="198" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A198" s="18"/>
       <c r="B198" s="18"/>
       <c r="C198" s="18"/>
@@ -15914,7 +15939,7 @@
       <c r="AF198" s="18"/>
       <c r="AG198" s="19"/>
     </row>
-    <row r="199" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:33" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A199" s="18"/>
       <c r="B199" s="18"/>
       <c r="C199" s="18"/>

</xml_diff>

<commit_message>
Card update part 2
</commit_message>
<xml_diff>
--- a/Master1.0.xlsx
+++ b/Master1.0.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="962" uniqueCount="576">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="994" uniqueCount="591">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -258,7 +258,7 @@
     <t xml:space="preserve">&lt;b&gt;&lt;i&gt;Behemoth&lt;/i&gt;&lt;/b&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">You can't be be forced to move against your will. When you move, declare one of your hex as your moving hex. Your other Hexes follow behind.  Moving through a 1 wide gap counts as moving 2 hexes.</t>
+    <t xml:space="preserve">You can't be be forced to move against your will.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;b&gt;&lt;i&gt;Massive Limbs&lt;/i&gt;&lt;/b&gt;</t>
@@ -267,10 +267,10 @@
     <t xml:space="preserve">Attacks that cost more than 2 AP cost 1 less and have &lt;b&gt;Reach&lt;/b&gt;.</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;b&gt;&lt;i&gt;Heft&lt;/i&gt;&lt;/b&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">After emergence, gain +1 Flesh.</t>
+    <t xml:space="preserve">&lt;b&gt;&lt;i&gt;Hefty&lt;/i&gt;&lt;/b&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">After emergence, gain +1 Heft.</t>
   </si>
   <si>
     <t xml:space="preserve">Glowing Kintsugi</t>
@@ -418,7 +418,7 @@
     <t xml:space="preserve">At the start of your turn, put a counter on an empty mode, then use that effect.</t>
   </si>
   <si>
-    <t xml:space="preserve"> </t>
+    <t xml:space="preserve">Mob of the Deep Ones</t>
   </si>
   <si>
     <t xml:space="preserve">hex1big   hex1big   hex1big</t>
@@ -545,10 +545,6 @@
     <t xml:space="preserve">Reduce damage from non-adjacent beings to 0.</t>
   </si>
   <si>
-    <t xml:space="preserve">You cannot be move or be made to move except with the move action.
-&lt;br /&gt;Moving into a 1 hex wide space counts as moving 2 hexes.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Unstable</t>
   </si>
   <si>
@@ -662,7 +658,7 @@
     <t xml:space="preserve">Your second attack each turn costs 1 less AP.</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;b&gt;&lt;i&gt;Creative Duelist&lt;/i&gt;&lt;/b&gt;</t>
+    <t xml:space="preserve">&lt;b&gt;&lt;i&gt;Creative Duellist&lt;/i&gt;&lt;/b&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">You may use Crit options available to any of your limbs on all attacks.</t>
@@ -1062,7 +1058,7 @@
     <t xml:space="preserve">Treacherous</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;b&gt;Snigger:&lt;/b&gt; WeirdT or &lt;b&gt;Exhasusted&lt;/b&gt;</t>
+    <t xml:space="preserve">&lt;b&gt;Snigger:&lt;/b&gt; WeirdT or &lt;b&gt;Exhausted&lt;/b&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">When you see a being take damage from a source other than you, you may increase that damage by 2. This does not stack.</t>
@@ -1319,7 +1315,7 @@
     <t xml:space="preserve">&lt;b&gt;Burst Block:&lt;/b&gt; Destroy this card</t>
   </si>
   <si>
-    <t xml:space="preserve">Completely block an incoming attack and deal 5 damage to all adjacent beings.</t>
+    <t xml:space="preserve">After taking damage, deal 6 damage to all adjacent beings.</t>
   </si>
   <si>
     <t xml:space="preserve">Explosive Polyps</t>
@@ -1426,7 +1422,7 @@
     <t xml:space="preserve">&lt;b&gt;Bloom:&lt;/b&gt;  WeirdT</t>
   </si>
   <si>
-    <t xml:space="preserve">Competely ignore damage from falling.</t>
+    <t xml:space="preserve">Completely ignore damage from falling.</t>
   </si>
   <si>
     <t xml:space="preserve">Lithium Geode</t>
@@ -1530,7 +1526,7 @@
     <t xml:space="preserve">&lt;b&gt;Snap:&lt;/b&gt; 3 AP + &lt;b&gt;Exhaust&lt;/b&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;b&gt;Damage = 6, Reach&lt;/b&gt;</t>
+    <t xml:space="preserve">&lt;b&gt;Damage = 7, Reach&lt;/b&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">Painted Slab</t>
@@ -1697,9 +1693,6 @@
   </si>
   <si>
     <t xml:space="preserve">&lt;b&gt;Smash:&lt;/b&gt; 3 AP + comptcompt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;b&gt;Damage = 7, Reach&lt;/b&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">Storm Conduit</t>
@@ -1800,6 +1793,86 @@
   <si>
     <t xml:space="preserve">&lt;b&gt;Damage = 5, Close&lt;/b&gt;
 &lt;br /&gt;Inflict the &lt;b&gt;Exhausted&lt;/b&gt; status effect on a hit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Effects from terrain or abilities cannot reduce your speed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fleet</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">While you have the &lt;b&gt;Well Rested&lt;/b&gt; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">status effect</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, gain an additional +1 speed.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Hands</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;b&gt;Anhedonia:&lt;/b&gt; 2 AP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Damage = 2, Close&lt;/b&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Handy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Terrain interactions cost 1 AP less.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Swarm of Eyes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;b&gt;Squint:&lt;/b&gt; 2 AP or (weirdT + 1 AP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Damage = 2, Ranged&lt;/b&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;b&gt;Armour Piercing:&lt;/b&gt; Damage from this attack can’t be reduced.
+&lt;br /&gt;&lt;b&gt;Insight:&lt;/b&gt; Regain a spent WeirdT.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spore Coat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Whenever you take damage, deal 1 damage to all adjacent beings. This damage can’t be reduced.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;b&gt;Sbonge:&lt;/b&gt; fleshTfleshT, &lt;b&gt;Exhausted&lt;/b&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Restore your composure.</t>
   </si>
 </sst>
 </file>
@@ -1809,7 +1882,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1838,6 +1911,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="11">
@@ -2942,7 +3021,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="68.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="66.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
         <v>50</v>
       </c>
@@ -3122,7 +3201,7 @@
         <v>31.2</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
         <v>66</v>
       </c>
@@ -3206,7 +3285,7 @@
         <v>31.2</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="46.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
         <v>72</v>
       </c>
@@ -4504,7 +4583,7 @@
         <v>57.6</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
         <v>164</v>
       </c>
@@ -4522,10 +4601,10 @@
         <v>35</v>
       </c>
       <c r="G22" s="11" t="s">
-        <v>165</v>
+        <v>75</v>
       </c>
       <c r="H22" s="11" t="s">
-        <v>166</v>
+        <v>76</v>
       </c>
       <c r="I22" s="10"/>
       <c r="J22" s="9" t="n">
@@ -4535,10 +4614,10 @@
         <v>35</v>
       </c>
       <c r="L22" s="11" t="s">
-        <v>167</v>
-      </c>
-      <c r="M22" s="9" t="s">
-        <v>168</v>
+        <v>165</v>
+      </c>
+      <c r="M22" s="11" t="s">
+        <v>166</v>
       </c>
       <c r="N22" s="12"/>
       <c r="O22" s="9" t="n">
@@ -4548,10 +4627,10 @@
         <v>35</v>
       </c>
       <c r="Q22" s="11" t="s">
-        <v>75</v>
+        <v>167</v>
       </c>
       <c r="R22" s="9" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="S22" s="10"/>
       <c r="T22" s="9"/>
@@ -4598,7 +4677,7 @@
     </row>
     <row r="23" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B23" s="8" t="s">
         <v>34</v>
@@ -4612,10 +4691,10 @@
         <v>35</v>
       </c>
       <c r="G23" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="H23" s="9" t="s">
         <v>171</v>
-      </c>
-      <c r="H23" s="9" t="s">
-        <v>172</v>
       </c>
       <c r="I23" s="18"/>
       <c r="J23" s="9" t="n">
@@ -4625,10 +4704,10 @@
         <v>35</v>
       </c>
       <c r="L23" s="11" t="s">
+        <v>172</v>
+      </c>
+      <c r="M23" s="9" t="s">
         <v>173</v>
-      </c>
-      <c r="M23" s="9" t="s">
-        <v>174</v>
       </c>
       <c r="N23" s="19"/>
       <c r="O23" s="9"/>
@@ -4690,7 +4769,7 @@
     </row>
     <row r="24" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B24" s="8" t="s">
         <v>34</v>
@@ -4704,10 +4783,10 @@
         <v>35</v>
       </c>
       <c r="G24" s="11" t="s">
+        <v>175</v>
+      </c>
+      <c r="H24" s="11" t="s">
         <v>176</v>
-      </c>
-      <c r="H24" s="11" t="s">
-        <v>177</v>
       </c>
       <c r="I24" s="10"/>
       <c r="J24" s="9" t="n">
@@ -4717,10 +4796,10 @@
         <v>38</v>
       </c>
       <c r="L24" s="11" t="s">
+        <v>177</v>
+      </c>
+      <c r="M24" s="11" t="s">
         <v>178</v>
-      </c>
-      <c r="M24" s="11" t="s">
-        <v>179</v>
       </c>
       <c r="N24" s="12"/>
       <c r="O24" s="11"/>
@@ -4772,13 +4851,13 @@
     </row>
     <row r="25" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B25" s="8" t="s">
         <v>34</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D25" s="10"/>
       <c r="E25" s="9" t="n">
@@ -4788,10 +4867,10 @@
         <v>38</v>
       </c>
       <c r="G25" s="11" t="s">
+        <v>181</v>
+      </c>
+      <c r="H25" s="11" t="s">
         <v>182</v>
-      </c>
-      <c r="H25" s="11" t="s">
-        <v>183</v>
       </c>
       <c r="I25" s="10"/>
       <c r="J25" s="9" t="n">
@@ -4801,10 +4880,10 @@
         <v>35</v>
       </c>
       <c r="L25" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="M25" s="9" t="s">
         <v>184</v>
-      </c>
-      <c r="M25" s="9" t="s">
-        <v>185</v>
       </c>
       <c r="N25" s="12"/>
       <c r="O25" s="9" t="n">
@@ -4814,10 +4893,10 @@
         <v>38</v>
       </c>
       <c r="Q25" s="11" t="s">
+        <v>185</v>
+      </c>
+      <c r="R25" s="9" t="s">
         <v>186</v>
-      </c>
-      <c r="R25" s="9" t="s">
-        <v>187</v>
       </c>
       <c r="S25" s="10"/>
       <c r="T25" s="9"/>
@@ -4864,7 +4943,7 @@
     </row>
     <row r="26" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B26" s="8" t="s">
         <v>34</v>
@@ -4878,10 +4957,10 @@
         <v>35</v>
       </c>
       <c r="G26" s="11" t="s">
+        <v>188</v>
+      </c>
+      <c r="H26" s="11" t="s">
         <v>189</v>
-      </c>
-      <c r="H26" s="11" t="s">
-        <v>190</v>
       </c>
       <c r="I26" s="10"/>
       <c r="J26" s="9" t="n">
@@ -4891,10 +4970,10 @@
         <v>35</v>
       </c>
       <c r="L26" s="11" t="s">
+        <v>190</v>
+      </c>
+      <c r="M26" s="9" t="s">
         <v>191</v>
-      </c>
-      <c r="M26" s="9" t="s">
-        <v>192</v>
       </c>
       <c r="N26" s="12"/>
       <c r="O26" s="9" t="n">
@@ -4904,10 +4983,10 @@
         <v>35</v>
       </c>
       <c r="Q26" s="11" t="s">
+        <v>192</v>
+      </c>
+      <c r="R26" s="13" t="s">
         <v>193</v>
-      </c>
-      <c r="R26" s="13" t="s">
-        <v>194</v>
       </c>
       <c r="S26" s="10"/>
       <c r="T26" s="9"/>
@@ -4954,7 +5033,7 @@
     </row>
     <row r="27" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B27" s="8" t="s">
         <v>34</v>
@@ -4968,10 +5047,10 @@
         <v>35</v>
       </c>
       <c r="G27" s="11" t="s">
+        <v>195</v>
+      </c>
+      <c r="H27" s="11" t="s">
         <v>196</v>
-      </c>
-      <c r="H27" s="11" t="s">
-        <v>197</v>
       </c>
       <c r="I27" s="10"/>
       <c r="J27" s="9" t="n">
@@ -4981,10 +5060,10 @@
         <v>38</v>
       </c>
       <c r="L27" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="M27" s="9" t="s">
         <v>198</v>
-      </c>
-      <c r="M27" s="9" t="s">
-        <v>199</v>
       </c>
       <c r="N27" s="12"/>
       <c r="O27" s="9"/>
@@ -5036,10 +5115,10 @@
     </row>
     <row r="28" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
+        <v>199</v>
+      </c>
+      <c r="B28" s="13" t="s">
         <v>200</v>
-      </c>
-      <c r="B28" s="13" t="s">
-        <v>201</v>
       </c>
       <c r="C28" s="9"/>
       <c r="D28" s="10"/>
@@ -5050,10 +5129,10 @@
         <v>38</v>
       </c>
       <c r="G28" s="11" t="s">
+        <v>201</v>
+      </c>
+      <c r="H28" s="11" t="s">
         <v>202</v>
-      </c>
-      <c r="H28" s="11" t="s">
-        <v>203</v>
       </c>
       <c r="I28" s="10"/>
       <c r="J28" s="9"/>
@@ -5110,10 +5189,10 @@
     </row>
     <row r="29" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B29" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C29" s="11"/>
       <c r="D29" s="10"/>
@@ -5124,10 +5203,10 @@
         <v>35</v>
       </c>
       <c r="G29" s="11" t="s">
+        <v>204</v>
+      </c>
+      <c r="H29" s="11" t="s">
         <v>205</v>
-      </c>
-      <c r="H29" s="11" t="s">
-        <v>206</v>
       </c>
       <c r="I29" s="10"/>
       <c r="J29" s="9" t="n">
@@ -5137,10 +5216,10 @@
         <v>35</v>
       </c>
       <c r="L29" s="9" t="s">
+        <v>206</v>
+      </c>
+      <c r="M29" s="9" t="s">
         <v>207</v>
-      </c>
-      <c r="M29" s="9" t="s">
-        <v>208</v>
       </c>
       <c r="N29" s="12"/>
       <c r="O29" s="9"/>
@@ -5192,10 +5271,10 @@
     </row>
     <row r="30" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C30" s="9"/>
       <c r="D30" s="18"/>
@@ -5206,10 +5285,10 @@
         <v>35</v>
       </c>
       <c r="G30" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="H30" s="9" t="s">
         <v>210</v>
-      </c>
-      <c r="H30" s="9" t="s">
-        <v>211</v>
       </c>
       <c r="I30" s="18"/>
       <c r="J30" s="9"/>
@@ -5266,10 +5345,10 @@
     </row>
     <row r="31" customFormat="false" ht="55.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C31" s="9"/>
       <c r="D31" s="18"/>
@@ -5280,10 +5359,10 @@
         <v>35</v>
       </c>
       <c r="G31" s="9" t="s">
+        <v>212</v>
+      </c>
+      <c r="H31" s="9" t="s">
         <v>213</v>
-      </c>
-      <c r="H31" s="9" t="s">
-        <v>214</v>
       </c>
       <c r="I31" s="18"/>
       <c r="J31" s="9"/>
@@ -5340,10 +5419,10 @@
     </row>
     <row r="32" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B32" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C32" s="9"/>
       <c r="D32" s="18"/>
@@ -5354,10 +5433,10 @@
         <v>35</v>
       </c>
       <c r="G32" s="9" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="I32" s="18"/>
       <c r="J32" s="9"/>
@@ -5414,10 +5493,10 @@
     </row>
     <row r="33" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C33" s="9"/>
       <c r="D33" s="18"/>
@@ -5428,10 +5507,10 @@
         <v>35</v>
       </c>
       <c r="G33" s="9" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H33" s="9" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="I33" s="18"/>
       <c r="J33" s="9"/>
@@ -5488,10 +5567,10 @@
     </row>
     <row r="34" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B34" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C34" s="9"/>
       <c r="D34" s="10"/>
@@ -5499,13 +5578,13 @@
         <v>1</v>
       </c>
       <c r="F34" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="G34" s="11" t="s">
         <v>220</v>
       </c>
-      <c r="G34" s="11" t="s">
+      <c r="H34" s="11" t="s">
         <v>221</v>
-      </c>
-      <c r="H34" s="11" t="s">
-        <v>222</v>
       </c>
       <c r="I34" s="10"/>
       <c r="J34" s="9"/>
@@ -5562,10 +5641,10 @@
     </row>
     <row r="35" customFormat="false" ht="55.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C35" s="9"/>
       <c r="D35" s="10"/>
@@ -5576,10 +5655,10 @@
         <v>35</v>
       </c>
       <c r="G35" s="11" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H35" s="11" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="I35" s="10"/>
       <c r="J35" s="9"/>
@@ -5636,10 +5715,10 @@
     </row>
     <row r="36" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B36" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C36" s="9"/>
       <c r="D36" s="10"/>
@@ -5650,10 +5729,10 @@
         <v>35</v>
       </c>
       <c r="G36" s="11" t="s">
+        <v>225</v>
+      </c>
+      <c r="H36" s="11" t="s">
         <v>226</v>
-      </c>
-      <c r="H36" s="11" t="s">
-        <v>227</v>
       </c>
       <c r="I36" s="10"/>
       <c r="J36" s="9" t="n">
@@ -5663,10 +5742,10 @@
         <v>35</v>
       </c>
       <c r="L36" s="11" t="s">
+        <v>227</v>
+      </c>
+      <c r="M36" s="9" t="s">
         <v>228</v>
-      </c>
-      <c r="M36" s="9" t="s">
-        <v>229</v>
       </c>
       <c r="N36" s="12"/>
       <c r="O36" s="9"/>
@@ -5718,10 +5797,10 @@
     </row>
     <row r="37" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C37" s="9"/>
       <c r="D37" s="10"/>
@@ -5732,10 +5811,10 @@
         <v>35</v>
       </c>
       <c r="G37" s="11" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H37" s="11" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="I37" s="10"/>
       <c r="J37" s="9"/>
@@ -5792,10 +5871,10 @@
     </row>
     <row r="38" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B38" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C38" s="9"/>
       <c r="D38" s="10"/>
@@ -5806,10 +5885,10 @@
         <v>35</v>
       </c>
       <c r="G38" s="11" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H38" s="11" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="I38" s="10"/>
       <c r="J38" s="9"/>
@@ -5866,13 +5945,13 @@
     </row>
     <row r="39" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="B39" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="C39" s="9" t="s">
         <v>234</v>
-      </c>
-      <c r="B39" s="13" t="s">
-        <v>201</v>
-      </c>
-      <c r="C39" s="9" t="s">
-        <v>235</v>
       </c>
       <c r="D39" s="10"/>
       <c r="E39" s="9" t="n">
@@ -5882,10 +5961,10 @@
         <v>38</v>
       </c>
       <c r="G39" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="H39" s="11" t="s">
         <v>236</v>
-      </c>
-      <c r="H39" s="11" t="s">
-        <v>237</v>
       </c>
       <c r="I39" s="10"/>
       <c r="J39" s="9"/>
@@ -5942,10 +6021,10 @@
     </row>
     <row r="40" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B40" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C40" s="9"/>
       <c r="D40" s="10"/>
@@ -5956,10 +6035,10 @@
         <v>38</v>
       </c>
       <c r="G40" s="11" t="s">
+        <v>238</v>
+      </c>
+      <c r="H40" s="11" t="s">
         <v>239</v>
-      </c>
-      <c r="H40" s="11" t="s">
-        <v>240</v>
       </c>
       <c r="I40" s="10"/>
       <c r="J40" s="9" t="n">
@@ -5969,10 +6048,10 @@
         <v>35</v>
       </c>
       <c r="L40" s="11" t="s">
+        <v>240</v>
+      </c>
+      <c r="M40" s="9" t="s">
         <v>241</v>
-      </c>
-      <c r="M40" s="9" t="s">
-        <v>242</v>
       </c>
       <c r="N40" s="12"/>
       <c r="O40" s="9"/>
@@ -6024,10 +6103,10 @@
     </row>
     <row r="41" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B41" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C41" s="9"/>
       <c r="D41" s="10"/>
@@ -6038,10 +6117,10 @@
         <v>35</v>
       </c>
       <c r="G41" s="11" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H41" s="11" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="I41" s="10"/>
       <c r="J41" s="9"/>
@@ -6098,10 +6177,10 @@
     </row>
     <row r="42" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B42" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C42" s="9"/>
       <c r="D42" s="10"/>
@@ -6112,10 +6191,10 @@
         <v>35</v>
       </c>
       <c r="G42" s="11" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H42" s="11" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="I42" s="10"/>
       <c r="J42" s="9"/>
@@ -6172,10 +6251,10 @@
     </row>
     <row r="43" customFormat="false" ht="55.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B43" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C43" s="9"/>
       <c r="D43" s="10"/>
@@ -6186,10 +6265,10 @@
         <v>35</v>
       </c>
       <c r="G43" s="11" t="s">
+        <v>247</v>
+      </c>
+      <c r="H43" s="11" t="s">
         <v>248</v>
-      </c>
-      <c r="H43" s="11" t="s">
-        <v>249</v>
       </c>
       <c r="I43" s="10"/>
       <c r="J43" s="9" t="n">
@@ -6199,10 +6278,10 @@
         <v>38</v>
       </c>
       <c r="L43" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="M43" s="9" t="s">
         <v>250</v>
-      </c>
-      <c r="M43" s="9" t="s">
-        <v>251</v>
       </c>
       <c r="N43" s="12"/>
       <c r="O43" s="9" t="n">
@@ -6212,10 +6291,10 @@
         <v>38</v>
       </c>
       <c r="Q43" s="11" t="s">
+        <v>251</v>
+      </c>
+      <c r="R43" s="9" t="s">
         <v>252</v>
-      </c>
-      <c r="R43" s="9" t="s">
-        <v>253</v>
       </c>
       <c r="S43" s="10"/>
       <c r="T43" s="9"/>
@@ -6262,10 +6341,10 @@
     </row>
     <row r="44" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B44" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C44" s="9"/>
       <c r="D44" s="10"/>
@@ -6276,10 +6355,10 @@
         <v>38</v>
       </c>
       <c r="G44" s="11" t="s">
+        <v>254</v>
+      </c>
+      <c r="H44" s="11" t="s">
         <v>255</v>
-      </c>
-      <c r="H44" s="11" t="s">
-        <v>256</v>
       </c>
       <c r="I44" s="10"/>
       <c r="J44" s="9" t="n">
@@ -6289,10 +6368,10 @@
         <v>35</v>
       </c>
       <c r="L44" s="11" t="s">
+        <v>256</v>
+      </c>
+      <c r="M44" s="11" t="s">
         <v>257</v>
-      </c>
-      <c r="M44" s="11" t="s">
-        <v>258</v>
       </c>
       <c r="N44" s="12"/>
       <c r="O44" s="9"/>
@@ -6344,26 +6423,26 @@
     </row>
     <row r="45" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="s">
+        <v>258</v>
+      </c>
+      <c r="B45" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="C45" s="9" t="s">
         <v>259</v>
-      </c>
-      <c r="B45" s="13" t="s">
-        <v>201</v>
-      </c>
-      <c r="C45" s="9" t="s">
-        <v>260</v>
       </c>
       <c r="D45" s="10"/>
       <c r="E45" s="9" t="n">
         <v>1</v>
       </c>
       <c r="F45" s="11" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G45" s="11" t="s">
+        <v>260</v>
+      </c>
+      <c r="H45" s="11" t="s">
         <v>261</v>
-      </c>
-      <c r="H45" s="11" t="s">
-        <v>262</v>
       </c>
       <c r="I45" s="10"/>
       <c r="J45" s="9"/>
@@ -6420,10 +6499,10 @@
     </row>
     <row r="46" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="7" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B46" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C46" s="9"/>
       <c r="D46" s="10"/>
@@ -6434,10 +6513,10 @@
         <v>35</v>
       </c>
       <c r="G46" s="11" t="s">
+        <v>263</v>
+      </c>
+      <c r="H46" s="11" t="s">
         <v>264</v>
-      </c>
-      <c r="H46" s="11" t="s">
-        <v>265</v>
       </c>
       <c r="I46" s="10"/>
       <c r="J46" s="9" t="n">
@@ -6447,10 +6526,10 @@
         <v>35</v>
       </c>
       <c r="L46" s="11" t="s">
+        <v>265</v>
+      </c>
+      <c r="M46" s="9" t="s">
         <v>266</v>
-      </c>
-      <c r="M46" s="9" t="s">
-        <v>267</v>
       </c>
       <c r="N46" s="12"/>
       <c r="O46" s="9"/>
@@ -6502,10 +6581,10 @@
     </row>
     <row r="47" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="7" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B47" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C47" s="9"/>
       <c r="D47" s="10"/>
@@ -6516,10 +6595,10 @@
         <v>35</v>
       </c>
       <c r="G47" s="11" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H47" s="11" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="I47" s="10"/>
       <c r="J47" s="9"/>
@@ -6576,10 +6655,10 @@
     </row>
     <row r="48" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B48" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C48" s="9"/>
       <c r="D48" s="10"/>
@@ -6590,10 +6669,10 @@
         <v>35</v>
       </c>
       <c r="G48" s="11" t="s">
+        <v>270</v>
+      </c>
+      <c r="H48" s="11" t="s">
         <v>271</v>
-      </c>
-      <c r="H48" s="11" t="s">
-        <v>272</v>
       </c>
       <c r="I48" s="10"/>
       <c r="J48" s="9" t="n">
@@ -6603,10 +6682,10 @@
         <v>38</v>
       </c>
       <c r="L48" s="11" t="s">
+        <v>272</v>
+      </c>
+      <c r="M48" s="9" t="s">
         <v>273</v>
-      </c>
-      <c r="M48" s="9" t="s">
-        <v>274</v>
       </c>
       <c r="N48" s="12"/>
       <c r="O48" s="9"/>
@@ -6658,10 +6737,10 @@
     </row>
     <row r="49" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="7" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B49" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C49" s="9"/>
       <c r="D49" s="10"/>
@@ -6672,10 +6751,10 @@
         <v>38</v>
       </c>
       <c r="G49" s="11" t="s">
+        <v>275</v>
+      </c>
+      <c r="H49" s="11" t="s">
         <v>276</v>
-      </c>
-      <c r="H49" s="11" t="s">
-        <v>277</v>
       </c>
       <c r="I49" s="10"/>
       <c r="J49" s="9"/>
@@ -6732,10 +6811,10 @@
     </row>
     <row r="50" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B50" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C50" s="9"/>
       <c r="D50" s="10"/>
@@ -6746,10 +6825,10 @@
         <v>35</v>
       </c>
       <c r="G50" s="11" t="s">
+        <v>278</v>
+      </c>
+      <c r="H50" s="11" t="s">
         <v>279</v>
-      </c>
-      <c r="H50" s="11" t="s">
-        <v>280</v>
       </c>
       <c r="I50" s="10"/>
       <c r="J50" s="9" t="n">
@@ -6759,10 +6838,10 @@
         <v>35</v>
       </c>
       <c r="L50" s="11" t="s">
+        <v>280</v>
+      </c>
+      <c r="M50" s="9" t="s">
         <v>281</v>
-      </c>
-      <c r="M50" s="9" t="s">
-        <v>282</v>
       </c>
       <c r="N50" s="12"/>
       <c r="O50" s="9"/>
@@ -6814,10 +6893,10 @@
     </row>
     <row r="51" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="7" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B51" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C51" s="9"/>
       <c r="D51" s="10"/>
@@ -6828,10 +6907,10 @@
         <v>38</v>
       </c>
       <c r="G51" s="11" t="s">
+        <v>283</v>
+      </c>
+      <c r="H51" s="11" t="s">
         <v>284</v>
-      </c>
-      <c r="H51" s="11" t="s">
-        <v>285</v>
       </c>
       <c r="I51" s="10"/>
       <c r="J51" s="9"/>
@@ -6888,10 +6967,10 @@
     </row>
     <row r="52" customFormat="false" ht="55.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B52" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C52" s="9"/>
       <c r="D52" s="10"/>
@@ -6902,10 +6981,10 @@
         <v>38</v>
       </c>
       <c r="G52" s="11" t="s">
+        <v>286</v>
+      </c>
+      <c r="H52" s="11" t="s">
         <v>287</v>
-      </c>
-      <c r="H52" s="11" t="s">
-        <v>288</v>
       </c>
       <c r="I52" s="10"/>
       <c r="J52" s="9"/>
@@ -6962,10 +7041,10 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B53" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C53" s="9"/>
       <c r="D53" s="10"/>
@@ -6976,10 +7055,10 @@
         <v>38</v>
       </c>
       <c r="G53" s="11" t="s">
+        <v>289</v>
+      </c>
+      <c r="H53" s="11" t="s">
         <v>290</v>
-      </c>
-      <c r="H53" s="11" t="s">
-        <v>291</v>
       </c>
       <c r="I53" s="10"/>
       <c r="J53" s="9"/>
@@ -7036,10 +7115,10 @@
     </row>
     <row r="54" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B54" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C54" s="9"/>
       <c r="D54" s="10"/>
@@ -7050,10 +7129,10 @@
         <v>38</v>
       </c>
       <c r="G54" s="11" t="s">
+        <v>292</v>
+      </c>
+      <c r="H54" s="11" t="s">
         <v>293</v>
-      </c>
-      <c r="H54" s="11" t="s">
-        <v>294</v>
       </c>
       <c r="I54" s="10"/>
       <c r="J54" s="9" t="n">
@@ -7063,10 +7142,10 @@
         <v>35</v>
       </c>
       <c r="L54" s="11" t="s">
+        <v>294</v>
+      </c>
+      <c r="M54" s="9" t="s">
         <v>295</v>
-      </c>
-      <c r="M54" s="9" t="s">
-        <v>296</v>
       </c>
       <c r="N54" s="12"/>
       <c r="O54" s="9"/>
@@ -7118,10 +7197,10 @@
     </row>
     <row r="55" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B55" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C55" s="9"/>
       <c r="D55" s="10"/>
@@ -7132,10 +7211,10 @@
         <v>35</v>
       </c>
       <c r="G55" s="11" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H55" s="11" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="I55" s="10"/>
       <c r="J55" s="9"/>
@@ -7192,10 +7271,10 @@
     </row>
     <row r="56" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="7" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B56" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C56" s="9"/>
       <c r="D56" s="10"/>
@@ -7206,10 +7285,10 @@
         <v>35</v>
       </c>
       <c r="G56" s="11" t="s">
+        <v>299</v>
+      </c>
+      <c r="H56" s="11" t="s">
         <v>300</v>
-      </c>
-      <c r="H56" s="11" t="s">
-        <v>301</v>
       </c>
       <c r="I56" s="10"/>
       <c r="J56" s="9" t="n">
@@ -7219,10 +7298,10 @@
         <v>38</v>
       </c>
       <c r="L56" s="11" t="s">
+        <v>301</v>
+      </c>
+      <c r="M56" s="9" t="s">
         <v>302</v>
-      </c>
-      <c r="M56" s="9" t="s">
-        <v>303</v>
       </c>
       <c r="N56" s="12"/>
       <c r="O56" s="9"/>
@@ -7274,10 +7353,10 @@
     </row>
     <row r="57" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="7" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B57" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C57" s="9"/>
       <c r="D57" s="10"/>
@@ -7288,10 +7367,10 @@
         <v>38</v>
       </c>
       <c r="G57" s="11" t="s">
+        <v>304</v>
+      </c>
+      <c r="H57" s="11" t="s">
         <v>305</v>
-      </c>
-      <c r="H57" s="11" t="s">
-        <v>306</v>
       </c>
       <c r="I57" s="10"/>
       <c r="J57" s="9" t="n">
@@ -7301,10 +7380,10 @@
         <v>35</v>
       </c>
       <c r="L57" s="11" t="s">
+        <v>306</v>
+      </c>
+      <c r="M57" s="9" t="s">
         <v>307</v>
-      </c>
-      <c r="M57" s="9" t="s">
-        <v>308</v>
       </c>
       <c r="N57" s="12"/>
       <c r="O57" s="9"/>
@@ -7356,10 +7435,10 @@
     </row>
     <row r="58" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="7" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B58" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C58" s="9"/>
       <c r="D58" s="10"/>
@@ -7370,23 +7449,23 @@
         <v>35</v>
       </c>
       <c r="G58" s="11" t="s">
+        <v>309</v>
+      </c>
+      <c r="H58" s="11" t="s">
         <v>310</v>
-      </c>
-      <c r="H58" s="11" t="s">
-        <v>311</v>
       </c>
       <c r="I58" s="10"/>
       <c r="J58" s="9" t="n">
         <v>5</v>
       </c>
       <c r="K58" s="11" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="L58" s="11" t="s">
+        <v>311</v>
+      </c>
+      <c r="M58" s="9" t="s">
         <v>312</v>
-      </c>
-      <c r="M58" s="9" t="s">
-        <v>313</v>
       </c>
       <c r="N58" s="12"/>
       <c r="O58" s="9"/>
@@ -7438,10 +7517,10 @@
     </row>
     <row r="59" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="7" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B59" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C59" s="9"/>
       <c r="D59" s="10"/>
@@ -7452,10 +7531,10 @@
         <v>35</v>
       </c>
       <c r="G59" s="11" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H59" s="11" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="I59" s="10"/>
       <c r="J59" s="9"/>
@@ -7512,10 +7591,10 @@
     </row>
     <row r="60" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="7" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B60" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C60" s="9"/>
       <c r="D60" s="10"/>
@@ -7526,10 +7605,10 @@
         <v>38</v>
       </c>
       <c r="G60" s="11" t="s">
+        <v>316</v>
+      </c>
+      <c r="H60" s="11" t="s">
         <v>317</v>
-      </c>
-      <c r="H60" s="11" t="s">
-        <v>318</v>
       </c>
       <c r="I60" s="10"/>
       <c r="J60" s="9" t="n">
@@ -7539,10 +7618,10 @@
         <v>35</v>
       </c>
       <c r="L60" s="11" t="s">
+        <v>318</v>
+      </c>
+      <c r="M60" s="9" t="s">
         <v>319</v>
-      </c>
-      <c r="M60" s="9" t="s">
-        <v>320</v>
       </c>
       <c r="N60" s="12"/>
       <c r="O60" s="9"/>
@@ -7594,10 +7673,10 @@
     </row>
     <row r="61" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="7" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B61" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C61" s="9"/>
       <c r="D61" s="10"/>
@@ -7608,10 +7687,10 @@
         <v>35</v>
       </c>
       <c r="G61" s="11" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H61" s="11" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="I61" s="10"/>
       <c r="J61" s="9"/>
@@ -7668,10 +7747,10 @@
     </row>
     <row r="62" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="7" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B62" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C62" s="9"/>
       <c r="D62" s="10"/>
@@ -7679,13 +7758,13 @@
         <v>1</v>
       </c>
       <c r="F62" s="11" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G62" s="11" t="s">
+        <v>323</v>
+      </c>
+      <c r="H62" s="11" t="s">
         <v>324</v>
-      </c>
-      <c r="H62" s="11" t="s">
-        <v>325</v>
       </c>
       <c r="I62" s="10"/>
       <c r="J62" s="9"/>
@@ -7742,10 +7821,10 @@
     </row>
     <row r="63" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="7" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B63" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C63" s="9"/>
       <c r="D63" s="10"/>
@@ -7753,13 +7832,13 @@
         <v>1</v>
       </c>
       <c r="F63" s="11" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G63" s="11" t="s">
+        <v>326</v>
+      </c>
+      <c r="H63" s="11" t="s">
         <v>327</v>
-      </c>
-      <c r="H63" s="11" t="s">
-        <v>328</v>
       </c>
       <c r="I63" s="10"/>
       <c r="J63" s="9"/>
@@ -7816,10 +7895,10 @@
     </row>
     <row r="64" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="7" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B64" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C64" s="9"/>
       <c r="D64" s="10"/>
@@ -7830,10 +7909,10 @@
         <v>38</v>
       </c>
       <c r="G64" s="11" t="s">
+        <v>329</v>
+      </c>
+      <c r="H64" s="11" t="s">
         <v>330</v>
-      </c>
-      <c r="H64" s="11" t="s">
-        <v>331</v>
       </c>
       <c r="I64" s="10"/>
       <c r="J64" s="9" t="n">
@@ -7843,10 +7922,10 @@
         <v>35</v>
       </c>
       <c r="L64" s="11" t="s">
+        <v>331</v>
+      </c>
+      <c r="M64" s="9" t="s">
         <v>332</v>
-      </c>
-      <c r="M64" s="9" t="s">
-        <v>333</v>
       </c>
       <c r="N64" s="12"/>
       <c r="O64" s="9"/>
@@ -7898,10 +7977,10 @@
     </row>
     <row r="65" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="7" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B65" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C65" s="9"/>
       <c r="D65" s="10"/>
@@ -7912,10 +7991,10 @@
         <v>35</v>
       </c>
       <c r="G65" s="11" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H65" s="11" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="I65" s="10"/>
       <c r="J65" s="9"/>
@@ -7972,10 +8051,10 @@
     </row>
     <row r="66" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="7" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B66" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C66" s="9"/>
       <c r="D66" s="10"/>
@@ -7983,13 +8062,13 @@
         <v>1</v>
       </c>
       <c r="F66" s="9" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G66" s="11" t="s">
+        <v>336</v>
+      </c>
+      <c r="H66" s="11" t="s">
         <v>337</v>
-      </c>
-      <c r="H66" s="11" t="s">
-        <v>338</v>
       </c>
       <c r="I66" s="10"/>
       <c r="J66" s="9" t="n">
@@ -7999,10 +8078,10 @@
         <v>35</v>
       </c>
       <c r="L66" s="9" t="s">
+        <v>338</v>
+      </c>
+      <c r="M66" s="9" t="s">
         <v>339</v>
-      </c>
-      <c r="M66" s="9" t="s">
-        <v>340</v>
       </c>
       <c r="N66" s="12"/>
       <c r="O66" s="9"/>
@@ -8054,10 +8133,10 @@
     </row>
     <row r="67" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="7" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="B67" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C67" s="9"/>
       <c r="D67" s="10"/>
@@ -8065,13 +8144,13 @@
         <v>1</v>
       </c>
       <c r="F67" s="11" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G67" s="11" t="s">
+        <v>341</v>
+      </c>
+      <c r="H67" s="11" t="s">
         <v>342</v>
-      </c>
-      <c r="H67" s="11" t="s">
-        <v>343</v>
       </c>
       <c r="I67" s="10"/>
       <c r="J67" s="9"/>
@@ -8128,10 +8207,10 @@
     </row>
     <row r="68" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="7" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="B68" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C68" s="9"/>
       <c r="D68" s="10"/>
@@ -8139,13 +8218,13 @@
         <v>1</v>
       </c>
       <c r="F68" s="11" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G68" s="11" t="s">
+        <v>344</v>
+      </c>
+      <c r="H68" s="11" t="s">
         <v>345</v>
-      </c>
-      <c r="H68" s="11" t="s">
-        <v>346</v>
       </c>
       <c r="I68" s="10"/>
       <c r="J68" s="9" t="n">
@@ -8155,10 +8234,10 @@
         <v>35</v>
       </c>
       <c r="L68" s="11" t="s">
+        <v>346</v>
+      </c>
+      <c r="M68" s="9" t="s">
         <v>347</v>
-      </c>
-      <c r="M68" s="9" t="s">
-        <v>348</v>
       </c>
       <c r="N68" s="12"/>
       <c r="O68" s="9"/>
@@ -8210,10 +8289,10 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="7" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B69" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C69" s="9"/>
       <c r="D69" s="10"/>
@@ -8224,10 +8303,10 @@
         <v>38</v>
       </c>
       <c r="G69" s="11" t="s">
+        <v>349</v>
+      </c>
+      <c r="H69" s="11" t="s">
         <v>350</v>
-      </c>
-      <c r="H69" s="11" t="s">
-        <v>351</v>
       </c>
       <c r="I69" s="10"/>
       <c r="J69" s="9"/>
@@ -8284,10 +8363,10 @@
     </row>
     <row r="70" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="7" t="s">
+        <v>351</v>
+      </c>
+      <c r="B70" s="20" t="s">
         <v>352</v>
-      </c>
-      <c r="B70" s="20" t="s">
-        <v>353</v>
       </c>
       <c r="C70" s="9"/>
       <c r="D70" s="18"/>
@@ -8298,10 +8377,10 @@
         <v>38</v>
       </c>
       <c r="G70" s="9" t="s">
+        <v>353</v>
+      </c>
+      <c r="H70" s="9" t="s">
         <v>354</v>
-      </c>
-      <c r="H70" s="9" t="s">
-        <v>355</v>
       </c>
       <c r="I70" s="18"/>
       <c r="J70" s="9" t="n">
@@ -8311,23 +8390,23 @@
         <v>74</v>
       </c>
       <c r="L70" s="9" t="s">
+        <v>355</v>
+      </c>
+      <c r="M70" s="9" t="s">
         <v>356</v>
-      </c>
-      <c r="M70" s="9" t="s">
-        <v>357</v>
       </c>
       <c r="N70" s="19"/>
       <c r="O70" s="9" t="n">
         <v>9.5</v>
       </c>
       <c r="P70" s="9" t="s">
+        <v>357</v>
+      </c>
+      <c r="Q70" s="9" t="s">
         <v>358</v>
       </c>
-      <c r="Q70" s="9" t="s">
+      <c r="R70" s="9" t="s">
         <v>359</v>
-      </c>
-      <c r="R70" s="9" t="s">
-        <v>360</v>
       </c>
       <c r="S70" s="18"/>
       <c r="T70" s="9"/>
@@ -8374,10 +8453,10 @@
     </row>
     <row r="71" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="7" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="B71" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C71" s="9"/>
       <c r="D71" s="18"/>
@@ -8388,23 +8467,23 @@
         <v>74</v>
       </c>
       <c r="G71" s="9" t="s">
+        <v>361</v>
+      </c>
+      <c r="H71" s="9" t="s">
         <v>362</v>
-      </c>
-      <c r="H71" s="9" t="s">
-        <v>363</v>
       </c>
       <c r="I71" s="18"/>
       <c r="J71" s="9" t="n">
         <v>9</v>
       </c>
       <c r="K71" s="9" t="s">
+        <v>357</v>
+      </c>
+      <c r="L71" s="9" t="s">
         <v>358</v>
       </c>
-      <c r="L71" s="9" t="s">
-        <v>359</v>
-      </c>
       <c r="M71" s="9" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="N71" s="19"/>
       <c r="O71" s="9" t="n">
@@ -8458,10 +8537,10 @@
     </row>
     <row r="72" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="7" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B72" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C72" s="9"/>
       <c r="D72" s="10"/>
@@ -8472,10 +8551,10 @@
         <v>38</v>
       </c>
       <c r="G72" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="H72" s="11" t="s">
         <v>366</v>
-      </c>
-      <c r="H72" s="11" t="s">
-        <v>367</v>
       </c>
       <c r="I72" s="10"/>
       <c r="J72" s="9" t="n">
@@ -8485,10 +8564,10 @@
         <v>38</v>
       </c>
       <c r="L72" s="9" t="s">
+        <v>367</v>
+      </c>
+      <c r="M72" s="9" t="s">
         <v>368</v>
-      </c>
-      <c r="M72" s="9" t="s">
-        <v>369</v>
       </c>
       <c r="N72" s="12"/>
       <c r="O72" s="9"/>
@@ -8540,10 +8619,10 @@
     </row>
     <row r="73" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="7" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B73" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C73" s="9"/>
       <c r="D73" s="18"/>
@@ -8554,10 +8633,10 @@
         <v>38</v>
       </c>
       <c r="G73" s="9" t="s">
+        <v>370</v>
+      </c>
+      <c r="H73" s="9" t="s">
         <v>371</v>
-      </c>
-      <c r="H73" s="9" t="s">
-        <v>372</v>
       </c>
       <c r="I73" s="18"/>
       <c r="J73" s="9" t="n">
@@ -8567,10 +8646,10 @@
         <v>38</v>
       </c>
       <c r="L73" s="9" t="s">
+        <v>372</v>
+      </c>
+      <c r="M73" s="9" t="s">
         <v>373</v>
-      </c>
-      <c r="M73" s="9" t="s">
-        <v>374</v>
       </c>
       <c r="N73" s="19"/>
       <c r="O73" s="9" t="n">
@@ -8624,10 +8703,10 @@
     </row>
     <row r="74" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="7" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="B74" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C74" s="9"/>
       <c r="D74" s="10"/>
@@ -8638,10 +8717,10 @@
         <v>38</v>
       </c>
       <c r="G74" s="11" t="s">
+        <v>375</v>
+      </c>
+      <c r="H74" s="11" t="s">
         <v>376</v>
-      </c>
-      <c r="H74" s="11" t="s">
-        <v>377</v>
       </c>
       <c r="I74" s="10"/>
       <c r="J74" s="9" t="n">
@@ -8651,10 +8730,10 @@
         <v>35</v>
       </c>
       <c r="L74" s="9" t="s">
+        <v>377</v>
+      </c>
+      <c r="M74" s="9" t="s">
         <v>378</v>
-      </c>
-      <c r="M74" s="9" t="s">
-        <v>379</v>
       </c>
       <c r="N74" s="12"/>
       <c r="O74" s="9"/>
@@ -8706,10 +8785,10 @@
     </row>
     <row r="75" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="7" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="B75" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C75" s="9"/>
       <c r="D75" s="10"/>
@@ -8720,10 +8799,10 @@
         <v>74</v>
       </c>
       <c r="G75" s="11" t="s">
+        <v>380</v>
+      </c>
+      <c r="H75" s="11" t="s">
         <v>381</v>
-      </c>
-      <c r="H75" s="11" t="s">
-        <v>382</v>
       </c>
       <c r="I75" s="10"/>
       <c r="J75" s="9" t="n">
@@ -8733,10 +8812,10 @@
         <v>35</v>
       </c>
       <c r="L75" s="11" t="s">
+        <v>382</v>
+      </c>
+      <c r="M75" s="9" t="s">
         <v>383</v>
-      </c>
-      <c r="M75" s="9" t="s">
-        <v>384</v>
       </c>
       <c r="N75" s="12"/>
       <c r="O75" s="9"/>
@@ -8788,10 +8867,10 @@
     </row>
     <row r="76" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="7" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="B76" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C76" s="9"/>
       <c r="D76" s="10"/>
@@ -8802,23 +8881,23 @@
         <v>74</v>
       </c>
       <c r="G76" s="11" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="H76" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="I76" s="10"/>
       <c r="J76" s="9" t="n">
         <v>9</v>
       </c>
       <c r="K76" s="9" t="s">
+        <v>357</v>
+      </c>
+      <c r="L76" s="9" t="s">
         <v>358</v>
       </c>
-      <c r="L76" s="9" t="s">
-        <v>359</v>
-      </c>
       <c r="M76" s="9" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="N76" s="12"/>
       <c r="O76" s="9"/>
@@ -8870,10 +8949,10 @@
     </row>
     <row r="77" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="7" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="B77" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C77" s="9"/>
       <c r="D77" s="10"/>
@@ -8884,10 +8963,10 @@
         <v>74</v>
       </c>
       <c r="G77" s="11" t="s">
+        <v>388</v>
+      </c>
+      <c r="H77" s="11" t="s">
         <v>389</v>
-      </c>
-      <c r="H77" s="11" t="s">
-        <v>390</v>
       </c>
       <c r="I77" s="10"/>
       <c r="J77" s="9" t="n">
@@ -8897,10 +8976,10 @@
         <v>35</v>
       </c>
       <c r="L77" s="9" t="s">
+        <v>390</v>
+      </c>
+      <c r="M77" s="9" t="s">
         <v>391</v>
-      </c>
-      <c r="M77" s="9" t="s">
-        <v>392</v>
       </c>
       <c r="N77" s="12"/>
       <c r="O77" s="9"/>
@@ -8952,10 +9031,10 @@
     </row>
     <row r="78" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="7" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B78" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C78" s="9"/>
       <c r="D78" s="10"/>
@@ -8966,10 +9045,10 @@
         <v>38</v>
       </c>
       <c r="G78" s="11" t="s">
+        <v>393</v>
+      </c>
+      <c r="H78" s="11" t="s">
         <v>394</v>
-      </c>
-      <c r="H78" s="11" t="s">
-        <v>395</v>
       </c>
       <c r="I78" s="10"/>
       <c r="J78" s="11" t="n">
@@ -8979,10 +9058,10 @@
         <v>35</v>
       </c>
       <c r="L78" s="9" t="s">
+        <v>395</v>
+      </c>
+      <c r="M78" s="9" t="s">
         <v>396</v>
-      </c>
-      <c r="M78" s="9" t="s">
-        <v>397</v>
       </c>
       <c r="N78" s="12"/>
       <c r="O78" s="9"/>
@@ -9034,10 +9113,10 @@
     </row>
     <row r="79" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="7" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="B79" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C79" s="9"/>
       <c r="D79" s="10"/>
@@ -9048,10 +9127,10 @@
         <v>74</v>
       </c>
       <c r="G79" s="11" t="s">
+        <v>398</v>
+      </c>
+      <c r="H79" s="11" t="s">
         <v>399</v>
-      </c>
-      <c r="H79" s="11" t="s">
-        <v>400</v>
       </c>
       <c r="I79" s="10"/>
       <c r="J79" s="9" t="n">
@@ -9061,10 +9140,10 @@
         <v>38</v>
       </c>
       <c r="L79" s="9" t="s">
+        <v>400</v>
+      </c>
+      <c r="M79" s="9" t="s">
         <v>401</v>
-      </c>
-      <c r="M79" s="9" t="s">
-        <v>402</v>
       </c>
       <c r="N79" s="12"/>
       <c r="O79" s="9"/>
@@ -9116,10 +9195,10 @@
     </row>
     <row r="80" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="7" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B80" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C80" s="9"/>
       <c r="D80" s="10"/>
@@ -9130,10 +9209,10 @@
         <v>74</v>
       </c>
       <c r="G80" s="11" t="s">
+        <v>403</v>
+      </c>
+      <c r="H80" s="11" t="s">
         <v>404</v>
-      </c>
-      <c r="H80" s="11" t="s">
-        <v>405</v>
       </c>
       <c r="I80" s="10"/>
       <c r="J80" s="11" t="n">
@@ -9143,23 +9222,23 @@
         <v>38</v>
       </c>
       <c r="L80" s="9" t="s">
+        <v>405</v>
+      </c>
+      <c r="M80" s="9" t="s">
         <v>406</v>
-      </c>
-      <c r="M80" s="9" t="s">
-        <v>407</v>
       </c>
       <c r="N80" s="12"/>
       <c r="O80" s="9" t="n">
         <v>9.5</v>
       </c>
       <c r="P80" s="9" t="s">
+        <v>357</v>
+      </c>
+      <c r="Q80" s="9" t="s">
         <v>358</v>
       </c>
-      <c r="Q80" s="9" t="s">
-        <v>359</v>
-      </c>
       <c r="R80" s="9" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="S80" s="10"/>
       <c r="T80" s="9"/>
@@ -9206,10 +9285,10 @@
     </row>
     <row r="81" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="7" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="B81" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C81" s="9"/>
       <c r="D81" s="10"/>
@@ -9220,10 +9299,10 @@
         <v>74</v>
       </c>
       <c r="G81" s="11" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="H81" s="11" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="I81" s="10"/>
       <c r="J81" s="9" t="n">
@@ -9233,23 +9312,23 @@
         <v>38</v>
       </c>
       <c r="L81" s="9" t="s">
+        <v>410</v>
+      </c>
+      <c r="M81" s="9" t="s">
         <v>411</v>
-      </c>
-      <c r="M81" s="9" t="s">
-        <v>412</v>
       </c>
       <c r="N81" s="12"/>
       <c r="O81" s="9" t="n">
         <v>9.5</v>
       </c>
       <c r="P81" s="9" t="s">
+        <v>357</v>
+      </c>
+      <c r="Q81" s="9" t="s">
         <v>358</v>
       </c>
-      <c r="Q81" s="9" t="s">
-        <v>359</v>
-      </c>
       <c r="R81" s="9" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="S81" s="10"/>
       <c r="T81" s="9"/>
@@ -9296,10 +9375,10 @@
     </row>
     <row r="82" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="7" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="B82" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C82" s="9"/>
       <c r="D82" s="10"/>
@@ -9310,10 +9389,10 @@
         <v>38</v>
       </c>
       <c r="G82" s="11" t="s">
+        <v>414</v>
+      </c>
+      <c r="H82" s="11" t="s">
         <v>415</v>
-      </c>
-      <c r="H82" s="11" t="s">
-        <v>416</v>
       </c>
       <c r="I82" s="10"/>
       <c r="J82" s="9" t="n">
@@ -9323,10 +9402,10 @@
         <v>74</v>
       </c>
       <c r="L82" s="9" t="s">
+        <v>416</v>
+      </c>
+      <c r="M82" s="9" t="s">
         <v>417</v>
-      </c>
-      <c r="M82" s="9" t="s">
-        <v>418</v>
       </c>
       <c r="N82" s="12"/>
       <c r="O82" s="9"/>
@@ -9378,10 +9457,10 @@
     </row>
     <row r="83" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="7" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="B83" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C83" s="9"/>
       <c r="D83" s="10"/>
@@ -9389,13 +9468,13 @@
         <v>1</v>
       </c>
       <c r="F83" s="11" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G83" s="11" t="s">
+        <v>419</v>
+      </c>
+      <c r="H83" s="11" t="s">
         <v>420</v>
-      </c>
-      <c r="H83" s="11" t="s">
-        <v>421</v>
       </c>
       <c r="I83" s="10"/>
       <c r="J83" s="9"/>
@@ -9452,13 +9531,13 @@
     </row>
     <row r="84" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="7" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="B84" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C84" s="9" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="D84" s="10"/>
       <c r="E84" s="9" t="n">
@@ -9468,23 +9547,23 @@
         <v>38</v>
       </c>
       <c r="G84" s="11" t="s">
+        <v>422</v>
+      </c>
+      <c r="H84" s="11" t="s">
         <v>423</v>
-      </c>
-      <c r="H84" s="11" t="s">
-        <v>424</v>
       </c>
       <c r="I84" s="10"/>
       <c r="J84" s="9" t="n">
         <v>4</v>
       </c>
       <c r="K84" s="9" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="L84" s="9" t="s">
+        <v>424</v>
+      </c>
+      <c r="M84" s="9" t="s">
         <v>425</v>
-      </c>
-      <c r="M84" s="9" t="s">
-        <v>426</v>
       </c>
       <c r="N84" s="12"/>
       <c r="O84" s="9"/>
@@ -9536,10 +9615,10 @@
     </row>
     <row r="85" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="7" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="B85" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C85" s="9"/>
       <c r="D85" s="10"/>
@@ -9550,23 +9629,23 @@
         <v>74</v>
       </c>
       <c r="G85" s="11" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="H85" s="11" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="I85" s="10"/>
       <c r="J85" s="11" t="n">
         <v>9.5</v>
       </c>
       <c r="K85" s="9" t="s">
+        <v>357</v>
+      </c>
+      <c r="L85" s="9" t="s">
         <v>358</v>
       </c>
-      <c r="L85" s="9" t="s">
-        <v>359</v>
-      </c>
       <c r="M85" s="9" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="N85" s="12"/>
       <c r="O85" s="9"/>
@@ -9618,10 +9697,10 @@
     </row>
     <row r="86" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="7" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="B86" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C86" s="9"/>
       <c r="D86" s="10"/>
@@ -9632,10 +9711,10 @@
         <v>74</v>
       </c>
       <c r="G86" s="11" t="s">
+        <v>430</v>
+      </c>
+      <c r="H86" s="11" t="s">
         <v>431</v>
-      </c>
-      <c r="H86" s="11" t="s">
-        <v>432</v>
       </c>
       <c r="I86" s="10"/>
       <c r="J86" s="9" t="n">
@@ -9645,23 +9724,23 @@
         <v>74</v>
       </c>
       <c r="L86" s="9" t="s">
+        <v>432</v>
+      </c>
+      <c r="M86" s="9" t="s">
         <v>433</v>
-      </c>
-      <c r="M86" s="9" t="s">
-        <v>434</v>
       </c>
       <c r="N86" s="12"/>
       <c r="O86" s="11" t="n">
         <v>9.5</v>
       </c>
       <c r="P86" s="9" t="s">
+        <v>357</v>
+      </c>
+      <c r="Q86" s="9" t="s">
         <v>358</v>
       </c>
-      <c r="Q86" s="9" t="s">
-        <v>359</v>
-      </c>
       <c r="R86" s="9" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="S86" s="10"/>
       <c r="T86" s="9"/>
@@ -9708,10 +9787,10 @@
     </row>
     <row r="87" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="7" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B87" s="21" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C87" s="11"/>
       <c r="D87" s="10"/>
@@ -9722,10 +9801,10 @@
         <v>74</v>
       </c>
       <c r="G87" s="11" t="s">
+        <v>435</v>
+      </c>
+      <c r="H87" s="11" t="s">
         <v>436</v>
-      </c>
-      <c r="H87" s="11" t="s">
-        <v>437</v>
       </c>
       <c r="I87" s="10"/>
       <c r="J87" s="9"/>
@@ -9782,10 +9861,10 @@
     </row>
     <row r="88" customFormat="false" ht="55.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="7" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="B88" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C88" s="9"/>
       <c r="D88" s="10"/>
@@ -9796,10 +9875,10 @@
         <v>74</v>
       </c>
       <c r="G88" s="11" t="s">
+        <v>438</v>
+      </c>
+      <c r="H88" s="11" t="s">
         <v>439</v>
-      </c>
-      <c r="H88" s="11" t="s">
-        <v>440</v>
       </c>
       <c r="I88" s="10"/>
       <c r="J88" s="9" t="n">
@@ -9809,10 +9888,10 @@
         <v>74</v>
       </c>
       <c r="L88" s="9" t="s">
+        <v>440</v>
+      </c>
+      <c r="M88" s="22" t="s">
         <v>441</v>
-      </c>
-      <c r="M88" s="22" t="s">
-        <v>442</v>
       </c>
       <c r="N88" s="12"/>
       <c r="O88" s="9"/>
@@ -9864,10 +9943,10 @@
     </row>
     <row r="89" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="7" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B89" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C89" s="11"/>
       <c r="D89" s="10"/>
@@ -9878,10 +9957,10 @@
         <v>74</v>
       </c>
       <c r="G89" s="11" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="H89" s="11" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="I89" s="10"/>
       <c r="J89" s="9" t="n">
@@ -9891,10 +9970,10 @@
         <v>38</v>
       </c>
       <c r="L89" s="9" t="s">
+        <v>444</v>
+      </c>
+      <c r="M89" s="9" t="s">
         <v>445</v>
-      </c>
-      <c r="M89" s="9" t="s">
-        <v>446</v>
       </c>
       <c r="N89" s="12"/>
       <c r="O89" s="9"/>
@@ -9946,10 +10025,10 @@
     </row>
     <row r="90" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="7" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="B90" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C90" s="9"/>
       <c r="D90" s="10"/>
@@ -9960,10 +10039,10 @@
         <v>74</v>
       </c>
       <c r="G90" s="11" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="H90" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="I90" s="10"/>
       <c r="J90" s="9" t="n">
@@ -9973,10 +10052,10 @@
         <v>74</v>
       </c>
       <c r="L90" s="9" t="s">
+        <v>448</v>
+      </c>
+      <c r="M90" s="9" t="s">
         <v>449</v>
-      </c>
-      <c r="M90" s="9" t="s">
-        <v>450</v>
       </c>
       <c r="N90" s="12"/>
       <c r="O90" s="9"/>
@@ -10028,10 +10107,10 @@
     </row>
     <row r="91" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="7" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="B91" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C91" s="9"/>
       <c r="D91" s="10"/>
@@ -10042,23 +10121,23 @@
         <v>74</v>
       </c>
       <c r="G91" s="11" t="s">
+        <v>451</v>
+      </c>
+      <c r="H91" s="11" t="s">
         <v>452</v>
-      </c>
-      <c r="H91" s="11" t="s">
-        <v>453</v>
       </c>
       <c r="I91" s="10"/>
       <c r="J91" s="9" t="n">
         <v>3</v>
       </c>
       <c r="K91" s="9" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="L91" s="9" t="s">
+        <v>453</v>
+      </c>
+      <c r="M91" s="9" t="s">
         <v>454</v>
-      </c>
-      <c r="M91" s="9" t="s">
-        <v>455</v>
       </c>
       <c r="N91" s="12"/>
       <c r="O91" s="9"/>
@@ -10110,13 +10189,13 @@
     </row>
     <row r="92" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="7" t="s">
+        <v>455</v>
+      </c>
+      <c r="B92" s="20" t="s">
+        <v>352</v>
+      </c>
+      <c r="C92" s="9" t="s">
         <v>456</v>
-      </c>
-      <c r="B92" s="20" t="s">
-        <v>353</v>
-      </c>
-      <c r="C92" s="9" t="s">
-        <v>457</v>
       </c>
       <c r="D92" s="10"/>
       <c r="E92" s="9" t="n">
@@ -10126,10 +10205,10 @@
         <v>38</v>
       </c>
       <c r="G92" s="11" t="s">
+        <v>457</v>
+      </c>
+      <c r="H92" s="11" t="s">
         <v>458</v>
-      </c>
-      <c r="H92" s="11" t="s">
-        <v>459</v>
       </c>
       <c r="I92" s="10"/>
       <c r="J92" s="9" t="n">
@@ -10139,10 +10218,10 @@
         <v>38</v>
       </c>
       <c r="L92" s="9" t="s">
+        <v>459</v>
+      </c>
+      <c r="M92" s="9" t="s">
         <v>460</v>
-      </c>
-      <c r="M92" s="9" t="s">
-        <v>461</v>
       </c>
       <c r="N92" s="12"/>
       <c r="O92" s="9"/>
@@ -10194,10 +10273,10 @@
     </row>
     <row r="93" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="7" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="B93" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C93" s="11"/>
       <c r="D93" s="10"/>
@@ -10208,10 +10287,10 @@
         <v>74</v>
       </c>
       <c r="G93" s="11" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="H93" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="I93" s="10"/>
       <c r="J93" s="9" t="n">
@@ -10221,10 +10300,10 @@
         <v>35</v>
       </c>
       <c r="L93" s="9" t="s">
+        <v>463</v>
+      </c>
+      <c r="M93" s="11" t="s">
         <v>464</v>
-      </c>
-      <c r="M93" s="11" t="s">
-        <v>465</v>
       </c>
       <c r="N93" s="12"/>
       <c r="O93" s="9"/>
@@ -10276,10 +10355,10 @@
     </row>
     <row r="94" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="7" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="B94" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C94" s="9"/>
       <c r="D94" s="10"/>
@@ -10290,10 +10369,10 @@
         <v>74</v>
       </c>
       <c r="G94" s="11" t="s">
+        <v>466</v>
+      </c>
+      <c r="H94" s="11" t="s">
         <v>467</v>
-      </c>
-      <c r="H94" s="11" t="s">
-        <v>468</v>
       </c>
       <c r="I94" s="10"/>
       <c r="J94" s="9" t="n">
@@ -10303,10 +10382,10 @@
         <v>35</v>
       </c>
       <c r="L94" s="9" t="s">
+        <v>468</v>
+      </c>
+      <c r="M94" s="9" t="s">
         <v>469</v>
-      </c>
-      <c r="M94" s="9" t="s">
-        <v>470</v>
       </c>
       <c r="N94" s="12"/>
       <c r="O94" s="9"/>
@@ -10358,10 +10437,10 @@
     </row>
     <row r="95" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="7" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="B95" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C95" s="9"/>
       <c r="D95" s="10"/>
@@ -10372,23 +10451,23 @@
         <v>74</v>
       </c>
       <c r="G95" s="11" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="H95" s="11" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="I95" s="10"/>
       <c r="J95" s="9" t="n">
         <v>10</v>
       </c>
       <c r="K95" s="9" t="s">
+        <v>357</v>
+      </c>
+      <c r="L95" s="9" t="s">
         <v>358</v>
       </c>
-      <c r="L95" s="9" t="s">
-        <v>359</v>
-      </c>
       <c r="M95" s="9" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="N95" s="12"/>
       <c r="O95" s="9"/>
@@ -10440,10 +10519,10 @@
     </row>
     <row r="96" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="7" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="B96" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C96" s="9"/>
       <c r="D96" s="10"/>
@@ -10451,13 +10530,13 @@
         <v>1</v>
       </c>
       <c r="F96" s="11" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G96" s="11" t="s">
+        <v>474</v>
+      </c>
+      <c r="H96" s="11" t="s">
         <v>475</v>
-      </c>
-      <c r="H96" s="11" t="s">
-        <v>476</v>
       </c>
       <c r="I96" s="10"/>
       <c r="J96" s="9" t="n">
@@ -10467,10 +10546,10 @@
         <v>35</v>
       </c>
       <c r="L96" s="9" t="s">
+        <v>476</v>
+      </c>
+      <c r="M96" s="9" t="s">
         <v>477</v>
-      </c>
-      <c r="M96" s="9" t="s">
-        <v>478</v>
       </c>
       <c r="N96" s="12"/>
       <c r="O96" s="9"/>
@@ -10522,10 +10601,10 @@
     </row>
     <row r="97" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="7" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="B97" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C97" s="9"/>
       <c r="D97" s="10"/>
@@ -10536,10 +10615,10 @@
         <v>74</v>
       </c>
       <c r="G97" s="11" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="H97" s="11" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="I97" s="10"/>
       <c r="J97" s="9" t="n">
@@ -10549,23 +10628,23 @@
         <v>35</v>
       </c>
       <c r="L97" s="9" t="s">
+        <v>480</v>
+      </c>
+      <c r="M97" s="9" t="s">
         <v>481</v>
-      </c>
-      <c r="M97" s="9" t="s">
-        <v>482</v>
       </c>
       <c r="N97" s="12"/>
       <c r="O97" s="9" t="n">
         <v>11</v>
       </c>
       <c r="P97" s="9" t="s">
+        <v>357</v>
+      </c>
+      <c r="Q97" s="9" t="s">
         <v>358</v>
       </c>
-      <c r="Q97" s="9" t="s">
-        <v>359</v>
-      </c>
       <c r="R97" s="9" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="S97" s="10"/>
       <c r="T97" s="9"/>
@@ -10612,10 +10691,10 @@
     </row>
     <row r="98" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="7" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="B98" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C98" s="9"/>
       <c r="D98" s="10"/>
@@ -10626,10 +10705,10 @@
         <v>74</v>
       </c>
       <c r="G98" s="11" t="s">
+        <v>484</v>
+      </c>
+      <c r="H98" s="11" t="s">
         <v>485</v>
-      </c>
-      <c r="H98" s="11" t="s">
-        <v>486</v>
       </c>
       <c r="I98" s="10"/>
       <c r="J98" s="9"/>
@@ -10686,10 +10765,10 @@
     </row>
     <row r="99" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="7" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="B99" s="21" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C99" s="11"/>
       <c r="D99" s="10"/>
@@ -10700,10 +10779,10 @@
         <v>74</v>
       </c>
       <c r="G99" s="11" t="s">
+        <v>487</v>
+      </c>
+      <c r="H99" s="11" t="s">
         <v>488</v>
-      </c>
-      <c r="H99" s="11" t="s">
-        <v>489</v>
       </c>
       <c r="I99" s="10"/>
       <c r="J99" s="9"/>
@@ -10760,10 +10839,10 @@
     </row>
     <row r="100" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="7" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="B100" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C100" s="9"/>
       <c r="D100" s="10"/>
@@ -10774,10 +10853,10 @@
         <v>74</v>
       </c>
       <c r="G100" s="11" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="H100" s="11" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="I100" s="10"/>
       <c r="J100" s="9" t="n">
@@ -10787,10 +10866,10 @@
         <v>38</v>
       </c>
       <c r="L100" s="9" t="s">
+        <v>491</v>
+      </c>
+      <c r="M100" s="9" t="s">
         <v>492</v>
-      </c>
-      <c r="M100" s="9" t="s">
-        <v>493</v>
       </c>
       <c r="N100" s="12"/>
       <c r="O100" s="9" t="n">
@@ -10800,10 +10879,10 @@
         <v>38</v>
       </c>
       <c r="Q100" s="9" t="s">
+        <v>493</v>
+      </c>
+      <c r="R100" s="9" t="s">
         <v>494</v>
-      </c>
-      <c r="R100" s="9" t="s">
-        <v>495</v>
       </c>
       <c r="S100" s="10"/>
       <c r="T100" s="9"/>
@@ -10850,10 +10929,10 @@
     </row>
     <row r="101" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="7" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B101" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C101" s="9"/>
       <c r="D101" s="10"/>
@@ -10864,23 +10943,23 @@
         <v>74</v>
       </c>
       <c r="G101" s="11" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="H101" s="11" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="I101" s="10"/>
       <c r="J101" s="9" t="n">
         <v>10</v>
       </c>
       <c r="K101" s="9" t="s">
+        <v>357</v>
+      </c>
+      <c r="L101" s="9" t="s">
         <v>358</v>
       </c>
-      <c r="L101" s="9" t="s">
-        <v>359</v>
-      </c>
       <c r="M101" s="9" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="N101" s="12"/>
       <c r="O101" s="9"/>
@@ -10932,10 +11011,10 @@
     </row>
     <row r="102" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="7" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="B102" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C102" s="9"/>
       <c r="D102" s="10"/>
@@ -10946,10 +11025,10 @@
         <v>74</v>
       </c>
       <c r="G102" s="11" t="s">
+        <v>499</v>
+      </c>
+      <c r="H102" s="11" t="s">
         <v>500</v>
-      </c>
-      <c r="H102" s="11" t="s">
-        <v>501</v>
       </c>
       <c r="I102" s="10"/>
       <c r="J102" s="9"/>
@@ -11006,10 +11085,10 @@
     </row>
     <row r="103" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="7" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="B103" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C103" s="9"/>
       <c r="D103" s="10"/>
@@ -11020,10 +11099,10 @@
         <v>38</v>
       </c>
       <c r="G103" s="11" t="s">
+        <v>502</v>
+      </c>
+      <c r="H103" s="11" t="s">
         <v>503</v>
-      </c>
-      <c r="H103" s="11" t="s">
-        <v>504</v>
       </c>
       <c r="I103" s="10"/>
       <c r="J103" s="9" t="n">
@@ -11033,10 +11112,10 @@
         <v>35</v>
       </c>
       <c r="L103" s="9" t="s">
+        <v>504</v>
+      </c>
+      <c r="M103" s="9" t="s">
         <v>505</v>
-      </c>
-      <c r="M103" s="9" t="s">
-        <v>506</v>
       </c>
       <c r="N103" s="12"/>
       <c r="O103" s="9"/>
@@ -11088,13 +11167,13 @@
     </row>
     <row r="104" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="7" t="s">
+        <v>506</v>
+      </c>
+      <c r="B104" s="21" t="s">
+        <v>352</v>
+      </c>
+      <c r="C104" s="11" t="s">
         <v>507</v>
-      </c>
-      <c r="B104" s="21" t="s">
-        <v>353</v>
-      </c>
-      <c r="C104" s="11" t="s">
-        <v>508</v>
       </c>
       <c r="D104" s="10"/>
       <c r="E104" s="9" t="n">
@@ -11104,10 +11183,10 @@
         <v>38</v>
       </c>
       <c r="G104" s="11" t="s">
+        <v>508</v>
+      </c>
+      <c r="H104" s="11" t="s">
         <v>509</v>
-      </c>
-      <c r="H104" s="11" t="s">
-        <v>510</v>
       </c>
       <c r="I104" s="10"/>
       <c r="J104" s="9" t="n">
@@ -11117,10 +11196,10 @@
         <v>35</v>
       </c>
       <c r="L104" s="9" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="M104" s="11" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="N104" s="12"/>
       <c r="O104" s="9"/>
@@ -11172,13 +11251,13 @@
     </row>
     <row r="105" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="7" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="B105" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C105" s="9" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="D105" s="10"/>
       <c r="E105" s="9" t="n">
@@ -11188,10 +11267,10 @@
         <v>74</v>
       </c>
       <c r="G105" s="11" t="s">
+        <v>512</v>
+      </c>
+      <c r="H105" s="11" t="s">
         <v>513</v>
-      </c>
-      <c r="H105" s="11" t="s">
-        <v>514</v>
       </c>
       <c r="I105" s="10"/>
       <c r="J105" s="9" t="n">
@@ -11201,10 +11280,10 @@
         <v>38</v>
       </c>
       <c r="L105" s="9" t="s">
+        <v>514</v>
+      </c>
+      <c r="M105" s="9" t="s">
         <v>515</v>
-      </c>
-      <c r="M105" s="9" t="s">
-        <v>516</v>
       </c>
       <c r="N105" s="12"/>
       <c r="O105" s="9"/>
@@ -11256,10 +11335,10 @@
     </row>
     <row r="106" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="7" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="B106" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C106" s="9"/>
       <c r="D106" s="10"/>
@@ -11270,10 +11349,10 @@
         <v>74</v>
       </c>
       <c r="G106" s="11" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="H106" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="I106" s="10"/>
       <c r="J106" s="9" t="n">
@@ -11283,23 +11362,23 @@
         <v>38</v>
       </c>
       <c r="L106" s="9" t="s">
+        <v>518</v>
+      </c>
+      <c r="M106" s="9" t="s">
         <v>519</v>
-      </c>
-      <c r="M106" s="9" t="s">
-        <v>520</v>
       </c>
       <c r="N106" s="12"/>
       <c r="O106" s="9" t="n">
         <v>10</v>
       </c>
       <c r="P106" s="9" t="s">
+        <v>357</v>
+      </c>
+      <c r="Q106" s="9" t="s">
         <v>358</v>
       </c>
-      <c r="Q106" s="9" t="s">
-        <v>359</v>
-      </c>
       <c r="R106" s="9" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="S106" s="10"/>
       <c r="T106" s="9"/>
@@ -11346,10 +11425,10 @@
     </row>
     <row r="107" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="7" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="B107" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C107" s="9"/>
       <c r="D107" s="10"/>
@@ -11360,23 +11439,23 @@
         <v>74</v>
       </c>
       <c r="G107" s="11" t="s">
+        <v>521</v>
+      </c>
+      <c r="H107" s="11" t="s">
         <v>522</v>
-      </c>
-      <c r="H107" s="11" t="s">
-        <v>523</v>
       </c>
       <c r="I107" s="10"/>
       <c r="J107" s="9" t="n">
         <v>10</v>
       </c>
       <c r="K107" s="9" t="s">
+        <v>357</v>
+      </c>
+      <c r="L107" s="9" t="s">
         <v>358</v>
       </c>
-      <c r="L107" s="9" t="s">
-        <v>359</v>
-      </c>
       <c r="M107" s="9" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="N107" s="12"/>
       <c r="O107" s="9"/>
@@ -11428,10 +11507,10 @@
     </row>
     <row r="108" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="7" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="B108" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C108" s="9"/>
       <c r="D108" s="18"/>
@@ -11442,10 +11521,10 @@
         <v>74</v>
       </c>
       <c r="G108" s="9" t="s">
+        <v>525</v>
+      </c>
+      <c r="H108" s="9" t="s">
         <v>526</v>
-      </c>
-      <c r="H108" s="9" t="s">
-        <v>527</v>
       </c>
       <c r="I108" s="18"/>
       <c r="J108" s="9" t="n">
@@ -11455,10 +11534,10 @@
         <v>35</v>
       </c>
       <c r="L108" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="M108" s="9" t="s">
         <v>528</v>
-      </c>
-      <c r="M108" s="9" t="s">
-        <v>529</v>
       </c>
       <c r="N108" s="19"/>
       <c r="O108" s="9" t="n">
@@ -11512,10 +11591,10 @@
     </row>
     <row r="109" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="7" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="B109" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C109" s="11"/>
       <c r="D109" s="10"/>
@@ -11526,23 +11605,23 @@
         <v>74</v>
       </c>
       <c r="G109" s="11" t="s">
+        <v>530</v>
+      </c>
+      <c r="H109" s="11" t="s">
         <v>531</v>
-      </c>
-      <c r="H109" s="11" t="s">
-        <v>532</v>
       </c>
       <c r="I109" s="10"/>
       <c r="J109" s="9" t="n">
         <v>9</v>
       </c>
       <c r="K109" s="9" t="s">
+        <v>357</v>
+      </c>
+      <c r="L109" s="9" t="s">
         <v>358</v>
       </c>
-      <c r="L109" s="9" t="s">
-        <v>359</v>
-      </c>
       <c r="M109" s="11" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="N109" s="12"/>
       <c r="O109" s="9"/>
@@ -11594,10 +11673,10 @@
     </row>
     <row r="110" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="7" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="B110" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C110" s="11"/>
       <c r="D110" s="10"/>
@@ -11608,23 +11687,23 @@
         <v>74</v>
       </c>
       <c r="G110" s="11" t="s">
+        <v>534</v>
+      </c>
+      <c r="H110" s="11" t="s">
         <v>535</v>
-      </c>
-      <c r="H110" s="11" t="s">
-        <v>536</v>
       </c>
       <c r="I110" s="10"/>
       <c r="J110" s="9" t="n">
         <v>10</v>
       </c>
       <c r="K110" s="9" t="s">
+        <v>357</v>
+      </c>
+      <c r="L110" s="9" t="s">
         <v>358</v>
       </c>
-      <c r="L110" s="9" t="s">
-        <v>359</v>
-      </c>
       <c r="M110" s="11" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="N110" s="12"/>
       <c r="O110" s="9"/>
@@ -11676,10 +11755,10 @@
     </row>
     <row r="111" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="7" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="B111" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C111" s="11"/>
       <c r="D111" s="10"/>
@@ -11690,23 +11769,23 @@
         <v>74</v>
       </c>
       <c r="G111" s="11" t="s">
+        <v>537</v>
+      </c>
+      <c r="H111" s="11" t="s">
         <v>538</v>
-      </c>
-      <c r="H111" s="11" t="s">
-        <v>539</v>
       </c>
       <c r="I111" s="10"/>
       <c r="J111" s="9" t="n">
         <v>9</v>
       </c>
       <c r="K111" s="9" t="s">
+        <v>357</v>
+      </c>
+      <c r="L111" s="9" t="s">
         <v>358</v>
       </c>
-      <c r="L111" s="9" t="s">
-        <v>359</v>
-      </c>
       <c r="M111" s="11" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="N111" s="12"/>
       <c r="O111" s="9"/>
@@ -11758,10 +11837,10 @@
     </row>
     <row r="112" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="7" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="B112" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C112" s="11"/>
       <c r="D112" s="10"/>
@@ -11772,10 +11851,10 @@
         <v>74</v>
       </c>
       <c r="G112" s="11" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="H112" s="11" t="s">
-        <v>543</v>
+        <v>488</v>
       </c>
       <c r="I112" s="10"/>
       <c r="J112" s="9"/>
@@ -11832,10 +11911,10 @@
     </row>
     <row r="113" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="7" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="B113" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C113" s="9"/>
       <c r="D113" s="10"/>
@@ -11846,10 +11925,10 @@
         <v>38</v>
       </c>
       <c r="G113" s="11" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="H113" s="11" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="I113" s="10"/>
       <c r="J113" s="9" t="n">
@@ -11859,10 +11938,10 @@
         <v>35</v>
       </c>
       <c r="L113" s="9" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="M113" s="9" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
       <c r="N113" s="12"/>
       <c r="O113" s="9" t="n">
@@ -11872,10 +11951,10 @@
         <v>35</v>
       </c>
       <c r="Q113" s="9" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
       <c r="R113" s="9" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="S113" s="10"/>
       <c r="T113" s="9"/>
@@ -11922,10 +12001,10 @@
     </row>
     <row r="114" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="7" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="B114" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C114" s="11"/>
       <c r="D114" s="10"/>
@@ -11936,10 +12015,10 @@
         <v>74</v>
       </c>
       <c r="G114" s="11" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="H114" s="11" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="I114" s="10"/>
       <c r="J114" s="9"/>
@@ -11996,10 +12075,10 @@
     </row>
     <row r="115" customFormat="false" ht="33.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="7" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="B115" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C115" s="11"/>
       <c r="D115" s="10"/>
@@ -12010,10 +12089,10 @@
         <v>38</v>
       </c>
       <c r="G115" s="11" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="H115" s="11" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
       <c r="I115" s="10"/>
       <c r="J115" s="9" t="n">
@@ -12023,10 +12102,10 @@
         <v>74</v>
       </c>
       <c r="L115" s="9" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="M115" s="11" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="N115" s="12"/>
       <c r="O115" s="9"/>
@@ -12078,10 +12157,10 @@
     </row>
     <row r="116" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="7" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="B116" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C116" s="11"/>
       <c r="D116" s="10"/>
@@ -12092,10 +12171,10 @@
         <v>74</v>
       </c>
       <c r="G116" s="11" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="H116" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="I116" s="10"/>
       <c r="J116" s="9" t="n">
@@ -12105,10 +12184,10 @@
         <v>35</v>
       </c>
       <c r="L116" s="9" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="M116" s="11" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="N116" s="12"/>
       <c r="O116" s="9"/>
@@ -12160,10 +12239,10 @@
     </row>
     <row r="117" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="7" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="B117" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C117" s="11"/>
       <c r="D117" s="10"/>
@@ -12174,36 +12253,36 @@
         <v>74</v>
       </c>
       <c r="G117" s="11" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="H117" s="11" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="I117" s="10"/>
       <c r="J117" s="9" t="n">
         <v>3</v>
       </c>
       <c r="K117" s="9" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="L117" s="9" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="M117" s="9" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="N117" s="12"/>
       <c r="O117" s="9" t="n">
         <v>10</v>
       </c>
       <c r="P117" s="9" t="s">
+        <v>357</v>
+      </c>
+      <c r="Q117" s="9" t="s">
         <v>358</v>
       </c>
-      <c r="Q117" s="9" t="s">
-        <v>359</v>
-      </c>
       <c r="R117" s="11" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="S117" s="10"/>
       <c r="T117" s="9"/>
@@ -12250,10 +12329,10 @@
     </row>
     <row r="118" customFormat="false" ht="44.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="7" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="B118" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C118" s="11"/>
       <c r="D118" s="10"/>
@@ -12264,10 +12343,10 @@
         <v>74</v>
       </c>
       <c r="G118" s="11" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="H118" s="11" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="I118" s="10"/>
       <c r="J118" s="9" t="n">
@@ -12277,10 +12356,10 @@
         <v>38</v>
       </c>
       <c r="L118" s="9" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="M118" s="9" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="N118" s="12"/>
       <c r="O118" s="9"/>
@@ -12332,10 +12411,10 @@
     </row>
     <row r="119" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="7" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="B119" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C119" s="11"/>
       <c r="D119" s="10"/>
@@ -12346,10 +12425,10 @@
         <v>74</v>
       </c>
       <c r="G119" s="11" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="H119" s="11" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="I119" s="10"/>
       <c r="J119" s="9"/>
@@ -12404,145 +12483,225 @@
         <v>31.2</v>
       </c>
     </row>
-    <row r="120" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A120" s="23"/>
-      <c r="B120" s="23"/>
-      <c r="C120" s="23"/>
-      <c r="D120" s="23"/>
-      <c r="E120" s="23"/>
-      <c r="F120" s="24"/>
-      <c r="G120" s="24"/>
-      <c r="H120" s="23"/>
-      <c r="I120" s="23"/>
-      <c r="J120" s="23"/>
-      <c r="K120" s="24"/>
-      <c r="L120" s="24"/>
-      <c r="M120" s="25"/>
-      <c r="N120" s="23"/>
-      <c r="O120" s="23"/>
-      <c r="P120" s="24"/>
-      <c r="Q120" s="24"/>
-      <c r="R120" s="23"/>
-      <c r="S120" s="23"/>
-      <c r="T120" s="23"/>
-      <c r="U120" s="23"/>
-      <c r="V120" s="23"/>
-      <c r="W120" s="23"/>
-      <c r="X120" s="23"/>
-      <c r="Y120" s="23"/>
-      <c r="Z120" s="23"/>
-      <c r="AA120" s="23"/>
-      <c r="AB120" s="23"/>
-      <c r="AC120" s="23"/>
-      <c r="AD120" s="23"/>
-      <c r="AE120" s="23"/>
-      <c r="AF120" s="23"/>
-      <c r="AG120" s="24"/>
-    </row>
-    <row r="121" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A121" s="23"/>
-      <c r="B121" s="23"/>
-      <c r="C121" s="23"/>
-      <c r="D121" s="23"/>
-      <c r="E121" s="23"/>
-      <c r="F121" s="24"/>
-      <c r="G121" s="24"/>
-      <c r="H121" s="23"/>
-      <c r="I121" s="23"/>
-      <c r="J121" s="23"/>
-      <c r="K121" s="24"/>
-      <c r="L121" s="24"/>
-      <c r="M121" s="25"/>
-      <c r="N121" s="23"/>
-      <c r="O121" s="23"/>
-      <c r="P121" s="24"/>
-      <c r="Q121" s="24"/>
-      <c r="R121" s="23"/>
-      <c r="S121" s="23"/>
-      <c r="T121" s="23"/>
-      <c r="U121" s="23"/>
-      <c r="V121" s="23"/>
-      <c r="W121" s="23"/>
-      <c r="X121" s="23"/>
-      <c r="Y121" s="23"/>
-      <c r="Z121" s="23"/>
-      <c r="AA121" s="23"/>
-      <c r="AB121" s="23"/>
-      <c r="AC121" s="23"/>
-      <c r="AD121" s="23"/>
-      <c r="AE121" s="23"/>
-      <c r="AF121" s="23"/>
-      <c r="AG121" s="24"/>
-    </row>
-    <row r="122" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A122" s="23"/>
-      <c r="B122" s="23"/>
-      <c r="C122" s="23"/>
-      <c r="D122" s="23"/>
-      <c r="E122" s="23"/>
-      <c r="F122" s="24"/>
-      <c r="G122" s="24"/>
-      <c r="H122" s="23"/>
-      <c r="I122" s="23"/>
-      <c r="J122" s="23"/>
-      <c r="K122" s="24"/>
-      <c r="L122" s="24"/>
-      <c r="M122" s="25"/>
-      <c r="N122" s="23"/>
-      <c r="O122" s="23"/>
-      <c r="P122" s="24"/>
-      <c r="Q122" s="24"/>
-      <c r="R122" s="23"/>
-      <c r="S122" s="23"/>
-      <c r="T122" s="23"/>
-      <c r="U122" s="23"/>
-      <c r="V122" s="23"/>
-      <c r="W122" s="23"/>
-      <c r="X122" s="23"/>
-      <c r="Y122" s="23"/>
-      <c r="Z122" s="23"/>
-      <c r="AA122" s="23"/>
-      <c r="AB122" s="23"/>
-      <c r="AC122" s="23"/>
-      <c r="AD122" s="23"/>
-      <c r="AE122" s="23"/>
-      <c r="AF122" s="23"/>
-      <c r="AG122" s="24"/>
-    </row>
-    <row r="123" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A123" s="23"/>
-      <c r="B123" s="23"/>
-      <c r="C123" s="23"/>
-      <c r="D123" s="23"/>
-      <c r="E123" s="23"/>
-      <c r="F123" s="24"/>
-      <c r="G123" s="24"/>
-      <c r="H123" s="23"/>
-      <c r="I123" s="23"/>
-      <c r="J123" s="23"/>
-      <c r="K123" s="24"/>
-      <c r="L123" s="24"/>
-      <c r="M123" s="25"/>
-      <c r="N123" s="23"/>
-      <c r="O123" s="23"/>
-      <c r="P123" s="24"/>
-      <c r="Q123" s="24"/>
-      <c r="R123" s="23"/>
-      <c r="S123" s="23"/>
-      <c r="T123" s="23"/>
-      <c r="U123" s="23"/>
-      <c r="V123" s="23"/>
-      <c r="W123" s="23"/>
-      <c r="X123" s="23"/>
-      <c r="Y123" s="23"/>
-      <c r="Z123" s="23"/>
-      <c r="AA123" s="23"/>
-      <c r="AB123" s="23"/>
-      <c r="AC123" s="23"/>
-      <c r="AD123" s="23"/>
-      <c r="AE123" s="23"/>
-      <c r="AF123" s="23"/>
-      <c r="AG123" s="24"/>
+    <row r="120" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="7" t="s">
+        <v>574</v>
+      </c>
+      <c r="B120" s="20" t="s">
+        <v>352</v>
+      </c>
+      <c r="C120" s="11"/>
+      <c r="D120" s="10"/>
+      <c r="E120" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F120" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="G120" s="11" t="s">
+        <v>346</v>
+      </c>
+      <c r="H120" s="11" t="s">
+        <v>575</v>
+      </c>
+      <c r="I120" s="10"/>
+      <c r="J120" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="K120" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="L120" s="9" t="s">
+        <v>576</v>
+      </c>
+      <c r="M120" s="9" t="s">
+        <v>577</v>
+      </c>
+      <c r="N120" s="12"/>
+      <c r="O120" s="9"/>
+      <c r="P120" s="9"/>
+      <c r="Q120" s="9"/>
+      <c r="R120" s="11"/>
+      <c r="S120" s="10"/>
+      <c r="T120" s="9"/>
+      <c r="U120" s="9"/>
+      <c r="V120" s="9"/>
+      <c r="W120" s="9"/>
+      <c r="X120" s="9"/>
+      <c r="Y120" s="9"/>
+      <c r="Z120" s="9"/>
+      <c r="AA120" s="9"/>
+      <c r="AB120" s="9"/>
+      <c r="AC120" s="9"/>
+      <c r="AD120" s="9"/>
+      <c r="AE120" s="9"/>
+      <c r="AF120" s="9"/>
+      <c r="AG120" s="11"/>
+    </row>
+    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A121" s="7" t="s">
+        <v>578</v>
+      </c>
+      <c r="B121" s="20" t="s">
+        <v>352</v>
+      </c>
+      <c r="C121" s="11"/>
+      <c r="D121" s="10"/>
+      <c r="E121" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F121" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="G121" s="11" t="s">
+        <v>579</v>
+      </c>
+      <c r="H121" s="11" t="s">
+        <v>580</v>
+      </c>
+      <c r="I121" s="10"/>
+      <c r="J121" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="K121" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="L121" s="9" t="s">
+        <v>581</v>
+      </c>
+      <c r="M121" s="9" t="s">
+        <v>582</v>
+      </c>
+      <c r="N121" s="12"/>
+      <c r="O121" s="9"/>
+      <c r="P121" s="9"/>
+      <c r="Q121" s="9"/>
+      <c r="R121" s="11"/>
+      <c r="S121" s="10"/>
+      <c r="T121" s="9"/>
+      <c r="U121" s="9"/>
+      <c r="V121" s="9"/>
+      <c r="W121" s="9"/>
+      <c r="X121" s="9"/>
+      <c r="Y121" s="9"/>
+      <c r="Z121" s="9"/>
+      <c r="AA121" s="9"/>
+      <c r="AB121" s="9"/>
+      <c r="AC121" s="9"/>
+      <c r="AD121" s="9"/>
+      <c r="AE121" s="9"/>
+      <c r="AF121" s="9"/>
+      <c r="AG121" s="11"/>
+    </row>
+    <row r="122" customFormat="false" ht="35.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A122" s="7" t="s">
+        <v>583</v>
+      </c>
+      <c r="B122" s="20" t="s">
+        <v>352</v>
+      </c>
+      <c r="C122" s="11"/>
+      <c r="D122" s="10"/>
+      <c r="E122" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F122" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="G122" s="11" t="s">
+        <v>584</v>
+      </c>
+      <c r="H122" s="11" t="s">
+        <v>585</v>
+      </c>
+      <c r="I122" s="10"/>
+      <c r="J122" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="K122" s="9" t="s">
+        <v>357</v>
+      </c>
+      <c r="L122" s="9" t="s">
+        <v>358</v>
+      </c>
+      <c r="M122" s="11" t="s">
+        <v>586</v>
+      </c>
+      <c r="N122" s="12"/>
+      <c r="O122" s="9"/>
+      <c r="P122" s="9"/>
+      <c r="Q122" s="9"/>
+      <c r="R122" s="11"/>
+      <c r="S122" s="10"/>
+      <c r="T122" s="9"/>
+      <c r="U122" s="9"/>
+      <c r="V122" s="9"/>
+      <c r="W122" s="9"/>
+      <c r="X122" s="9"/>
+      <c r="Y122" s="9"/>
+      <c r="Z122" s="9"/>
+      <c r="AA122" s="9"/>
+      <c r="AB122" s="9"/>
+      <c r="AC122" s="9"/>
+      <c r="AD122" s="9"/>
+      <c r="AE122" s="9"/>
+      <c r="AF122" s="9"/>
+      <c r="AG122" s="11"/>
+    </row>
+    <row r="123" customFormat="false" ht="22.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A123" s="7" t="s">
+        <v>587</v>
+      </c>
+      <c r="B123" s="20" t="s">
+        <v>352</v>
+      </c>
+      <c r="C123" s="11"/>
+      <c r="D123" s="10"/>
+      <c r="E123" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F123" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="G123" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="H123" s="11" t="s">
+        <v>588</v>
+      </c>
+      <c r="I123" s="10"/>
+      <c r="J123" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="K123" s="9" t="s">
+        <v>219</v>
+      </c>
+      <c r="L123" s="9" t="s">
+        <v>589</v>
+      </c>
+      <c r="M123" s="11" t="s">
+        <v>590</v>
+      </c>
+      <c r="N123" s="12"/>
+      <c r="O123" s="9"/>
+      <c r="P123" s="9"/>
+      <c r="Q123" s="9"/>
+      <c r="R123" s="11"/>
+      <c r="S123" s="10"/>
+      <c r="T123" s="9"/>
+      <c r="U123" s="9"/>
+      <c r="V123" s="9"/>
+      <c r="W123" s="9"/>
+      <c r="X123" s="9"/>
+      <c r="Y123" s="9"/>
+      <c r="Z123" s="9"/>
+      <c r="AA123" s="9"/>
+      <c r="AB123" s="9"/>
+      <c r="AC123" s="9"/>
+      <c r="AD123" s="9"/>
+      <c r="AE123" s="9"/>
+      <c r="AF123" s="9"/>
+      <c r="AG123" s="11"/>
     </row>
     <row r="124" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="23"/>
@@ -15188,21 +15347,21 @@
       <formula>NOT(ISERROR(SEARCH("Spell",B2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B120:B198">
+  <conditionalFormatting sqref="B124:B198">
     <cfRule type="containsText" priority="7" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="Accessory" dxfId="17">
-      <formula>NOT(ISERROR(SEARCH("Accessory",B120)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Accessory",B124)))</formula>
     </cfRule>
     <cfRule type="containsText" priority="8" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="Armour" dxfId="18">
-      <formula>NOT(ISERROR(SEARCH("Armour",B120)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Armour",B124)))</formula>
     </cfRule>
     <cfRule type="containsText" priority="9" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="Equipment" dxfId="19">
-      <formula>NOT(ISERROR(SEARCH("Equipment",B120)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Equipment",B124)))</formula>
     </cfRule>
     <cfRule type="containsText" priority="10" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="Impression" dxfId="20">
-      <formula>NOT(ISERROR(SEARCH("Impression",B120)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Impression",B124)))</formula>
     </cfRule>
     <cfRule type="containsText" priority="11" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="Spell" dxfId="21">
-      <formula>NOT(ISERROR(SEARCH("Spell",B120)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Spell",B124)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C17">

</xml_diff>

<commit_message>
Text white borders gone!
</commit_message>
<xml_diff>
--- a/Master1.0.xlsx
+++ b/Master1.0.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kage\Documents\GitHub\Sculpt\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kagen\OneDrive\Documents\GitHub\Sculpt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{381C4C9F-CB23-41AE-A0D0-36151F81A6B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D64EC32A-1366-4275-9155-350ABBB028DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet3" sheetId="1" r:id="rId1"/>
@@ -2167,7 +2167,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Pūnoa" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2427,33 +2427,33 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AI201"/>
-  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="11" customWidth="1"/>
     <col min="3" max="4" width="10" customWidth="1"/>
-    <col min="5" max="5" width="17.140625" customWidth="1"/>
-    <col min="6" max="6" width="1.42578125" customWidth="1"/>
-    <col min="7" max="7" width="4.28515625" customWidth="1"/>
-    <col min="8" max="8" width="8.28515625" customWidth="1"/>
+    <col min="5" max="5" width="17.109375" customWidth="1"/>
+    <col min="6" max="6" width="1.44140625" customWidth="1"/>
+    <col min="7" max="7" width="4.33203125" customWidth="1"/>
+    <col min="8" max="8" width="8.33203125" customWidth="1"/>
     <col min="9" max="9" width="33" customWidth="1"/>
-    <col min="10" max="10" width="42.42578125" customWidth="1"/>
-    <col min="11" max="11" width="1.42578125" customWidth="1"/>
-    <col min="12" max="12" width="6.85546875" customWidth="1"/>
-    <col min="13" max="13" width="14.85546875" customWidth="1"/>
-    <col min="14" max="14" width="31.7109375" customWidth="1"/>
-    <col min="15" max="15" width="37.85546875" style="1" customWidth="1"/>
-    <col min="16" max="16" width="1.42578125" customWidth="1"/>
-    <col min="17" max="17" width="6.5703125" customWidth="1"/>
-    <col min="18" max="18" width="8.42578125" customWidth="1"/>
-    <col min="19" max="19" width="25.5703125" customWidth="1"/>
-    <col min="20" max="20" width="35.140625" customWidth="1"/>
-    <col min="21" max="21" width="1.42578125" customWidth="1"/>
+    <col min="10" max="10" width="42.44140625" customWidth="1"/>
+    <col min="11" max="11" width="1.44140625" customWidth="1"/>
+    <col min="12" max="12" width="6.88671875" customWidth="1"/>
+    <col min="13" max="13" width="14.88671875" customWidth="1"/>
+    <col min="14" max="14" width="31.6640625" customWidth="1"/>
+    <col min="15" max="15" width="37.88671875" style="1" customWidth="1"/>
+    <col min="16" max="16" width="1.44140625" customWidth="1"/>
+    <col min="17" max="17" width="6.5546875" customWidth="1"/>
+    <col min="18" max="18" width="8.44140625" customWidth="1"/>
+    <col min="19" max="19" width="25.5546875" customWidth="1"/>
+    <col min="20" max="20" width="35.109375" customWidth="1"/>
+    <col min="21" max="21" width="1.44140625" customWidth="1"/>
     <col min="22" max="22" width="10" customWidth="1"/>
     <col min="23" max="23" width="38" customWidth="1"/>
-    <col min="26" max="33" width="10.5703125" customWidth="1"/>
+    <col min="26" max="33" width="10.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2560,7 +2560,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:35" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2666,7 +2666,7 @@
         <v>62.800000000000004</v>
       </c>
     </row>
-    <row r="3" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
@@ -2762,7 +2762,7 @@
         <v>58.400000000000006</v>
       </c>
     </row>
-    <row r="4" spans="1:35" ht="90" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>1</v>
       </c>
@@ -2862,7 +2862,7 @@
         <v>71.599999999999994</v>
       </c>
     </row>
-    <row r="5" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>1</v>
       </c>
@@ -2954,7 +2954,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="6" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>1</v>
       </c>
@@ -3044,7 +3044,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="7" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>1</v>
       </c>
@@ -3142,7 +3142,7 @@
         <v>58.400000000000006</v>
       </c>
     </row>
-    <row r="8" spans="1:35" ht="90" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:35" ht="72" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>1</v>
       </c>
@@ -3230,7 +3230,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="9" spans="1:35" ht="60" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:35" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>1</v>
       </c>
@@ -3326,7 +3326,7 @@
         <v>62.800000000000004</v>
       </c>
     </row>
-    <row r="10" spans="1:35" ht="60" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:35" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>1</v>
       </c>
@@ -3414,7 +3414,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="11" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>1</v>
       </c>
@@ -3512,7 +3512,7 @@
         <v>49.6</v>
       </c>
     </row>
-    <row r="12" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>1</v>
       </c>
@@ -3600,7 +3600,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="13" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>1</v>
       </c>
@@ -3688,7 +3688,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="14" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>1</v>
       </c>
@@ -3784,7 +3784,7 @@
         <v>62.800000000000004</v>
       </c>
     </row>
-    <row r="15" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>1</v>
       </c>
@@ -3882,7 +3882,7 @@
         <v>58.400000000000006</v>
       </c>
     </row>
-    <row r="16" spans="1:35" ht="120" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:35" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>1</v>
       </c>
@@ -3970,7 +3970,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="17" spans="1:35" ht="60" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:35" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>1</v>
       </c>
@@ -4068,7 +4068,7 @@
         <v>67.2</v>
       </c>
     </row>
-    <row r="18" spans="1:35" ht="60" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:35" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>1</v>
       </c>
@@ -4164,7 +4164,7 @@
         <v>67.2</v>
       </c>
     </row>
-    <row r="19" spans="1:35" ht="60" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>1</v>
       </c>
@@ -4260,7 +4260,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="20" spans="1:35" ht="60" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:35" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>1</v>
       </c>
@@ -4348,7 +4348,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="21" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>1</v>
       </c>
@@ -4436,7 +4436,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="22" spans="1:35" ht="135" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:35" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>1</v>
       </c>
@@ -4536,7 +4536,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="23" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>1</v>
       </c>
@@ -4634,7 +4634,7 @@
         <v>58.400000000000006</v>
       </c>
     </row>
-    <row r="24" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>1</v>
       </c>
@@ -4722,7 +4722,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="25" spans="1:35" ht="60" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:35" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>1</v>
       </c>
@@ -4810,7 +4810,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="26" spans="1:35" ht="60" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:35" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>1</v>
       </c>
@@ -4908,7 +4908,7 @@
         <v>67.2</v>
       </c>
     </row>
-    <row r="27" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>1</v>
       </c>
@@ -5004,7 +5004,7 @@
         <v>62.800000000000004</v>
       </c>
     </row>
-    <row r="28" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>1</v>
       </c>
@@ -5092,7 +5092,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="29" spans="1:35" ht="60" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>1</v>
       </c>
@@ -5172,7 +5172,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="30" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>1</v>
       </c>
@@ -5249,7 +5249,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="31" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>1</v>
       </c>
@@ -5329,7 +5329,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="32" spans="1:35" ht="75" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:35" ht="72" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>1</v>
       </c>
@@ -5409,7 +5409,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="33" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>1</v>
       </c>
@@ -5489,7 +5489,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="34" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>1</v>
       </c>
@@ -5569,7 +5569,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="35" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>1</v>
       </c>
@@ -5649,7 +5649,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="36" spans="1:35" ht="75" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:35" ht="72" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>1</v>
       </c>
@@ -5729,7 +5729,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="37" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>1</v>
       </c>
@@ -5817,7 +5817,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="38" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>1</v>
       </c>
@@ -5897,7 +5897,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="39" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>1</v>
       </c>
@@ -5977,7 +5977,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="40" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>1</v>
       </c>
@@ -6057,7 +6057,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="41" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>1</v>
       </c>
@@ -6139,7 +6139,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="42" spans="1:35" ht="75" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>1</v>
       </c>
@@ -6227,7 +6227,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="43" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>1</v>
       </c>
@@ -6307,7 +6307,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="44" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>1</v>
       </c>
@@ -6387,7 +6387,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="45" spans="1:35" ht="90" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:35" ht="72" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>1</v>
       </c>
@@ -6483,7 +6483,7 @@
         <v>62.800000000000004</v>
       </c>
     </row>
-    <row r="46" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>1</v>
       </c>
@@ -6571,7 +6571,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="47" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>1</v>
       </c>
@@ -6653,7 +6653,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="48" spans="1:35" ht="60" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>1</v>
       </c>
@@ -6741,7 +6741,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="49" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>1</v>
       </c>
@@ -6821,7 +6821,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="50" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>1</v>
       </c>
@@ -6909,7 +6909,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="51" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>1</v>
       </c>
@@ -6989,7 +6989,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="52" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>1</v>
       </c>
@@ -7069,7 +7069,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="53" spans="1:35" ht="90" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:35" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>1</v>
       </c>
@@ -7149,7 +7149,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="54" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>1</v>
       </c>
@@ -7229,7 +7229,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="55" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>1</v>
       </c>
@@ -7317,7 +7317,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="56" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>1</v>
       </c>
@@ -7397,7 +7397,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="57" spans="1:35" ht="60" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>1</v>
       </c>
@@ -7485,7 +7485,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="58" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>1</v>
       </c>
@@ -7573,7 +7573,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="59" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>1</v>
       </c>
@@ -7661,7 +7661,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="60" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>1</v>
       </c>
@@ -7741,7 +7741,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="61" spans="1:35" ht="75" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:35" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>1</v>
       </c>
@@ -7829,7 +7829,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="62" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>1</v>
       </c>
@@ -7909,7 +7909,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="63" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>1</v>
       </c>
@@ -7989,7 +7989,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="64" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>1</v>
       </c>
@@ -8069,7 +8069,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="65" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>1</v>
       </c>
@@ -8157,7 +8157,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="66" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>1</v>
       </c>
@@ -8237,7 +8237,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="67" spans="1:35" ht="60" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>1</v>
       </c>
@@ -8325,7 +8325,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="68" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>1</v>
       </c>
@@ -8413,7 +8413,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="69" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>1</v>
       </c>
@@ -8493,7 +8493,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="70" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>1</v>
       </c>
@@ -8573,7 +8573,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="71" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>1</v>
       </c>
@@ -8669,7 +8669,7 @@
         <v>69.400000000000006</v>
       </c>
     </row>
-    <row r="72" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>1</v>
       </c>
@@ -8759,7 +8759,7 @@
         <v>49.6</v>
       </c>
     </row>
-    <row r="73" spans="1:35" ht="60" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>1</v>
       </c>
@@ -8847,7 +8847,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="74" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>1</v>
       </c>
@@ -8929,7 +8929,7 @@
         <v>49.6</v>
       </c>
     </row>
-    <row r="75" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>1</v>
       </c>
@@ -9017,7 +9017,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="76" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>1</v>
       </c>
@@ -9105,7 +9105,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="77" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>1</v>
       </c>
@@ -9193,7 +9193,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="78" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>1</v>
       </c>
@@ -9281,7 +9281,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="79" spans="1:35" ht="75" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:35" ht="72" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>1</v>
       </c>
@@ -9371,7 +9371,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="80" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>1</v>
       </c>
@@ -9459,7 +9459,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="81" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>1</v>
       </c>
@@ -9555,7 +9555,7 @@
         <v>71.599999999999994</v>
       </c>
     </row>
-    <row r="82" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>1</v>
       </c>
@@ -9643,7 +9643,7 @@
         <v>69.400000000000006</v>
       </c>
     </row>
-    <row r="83" spans="1:35" ht="60" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:35" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>1</v>
       </c>
@@ -9739,7 +9739,7 @@
         <v>67.2</v>
       </c>
     </row>
-    <row r="84" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>1</v>
       </c>
@@ -9827,7 +9827,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="85" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>1</v>
       </c>
@@ -9915,7 +9915,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="86" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>1</v>
       </c>
@@ -10003,7 +10003,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="87" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>1</v>
       </c>
@@ -10101,7 +10101,7 @@
         <v>58.400000000000006</v>
       </c>
     </row>
-    <row r="88" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>1</v>
       </c>
@@ -10199,7 +10199,7 @@
         <v>49.6</v>
       </c>
     </row>
-    <row r="89" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>1</v>
       </c>
@@ -10287,7 +10287,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="90" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>1</v>
       </c>
@@ -10383,7 +10383,7 @@
         <v>71.599999999999994</v>
       </c>
     </row>
-    <row r="91" spans="1:35" ht="60" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>1</v>
       </c>
@@ -10463,7 +10463,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="92" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>1</v>
       </c>
@@ -10559,7 +10559,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="93" spans="1:35" ht="75" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:35" ht="72" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>1</v>
       </c>
@@ -10647,7 +10647,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="94" spans="1:35" ht="75" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:35" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>1</v>
       </c>
@@ -10735,7 +10735,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="95" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>1</v>
       </c>
@@ -10823,7 +10823,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="96" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>1</v>
       </c>
@@ -10913,7 +10913,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="97" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>1</v>
       </c>
@@ -11001,7 +11001,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="98" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>1</v>
       </c>
@@ -11053,11 +11053,11 @@
       <c r="Y98" s="8"/>
       <c r="Z98" s="8"/>
       <c r="AA98" s="8">
-        <f t="shared" ref="AA98:AA129" si="27">AC98+Z$2</f>
+        <f t="shared" ref="AA98:AA127" si="27">AC98+Z$2</f>
         <v>20</v>
       </c>
       <c r="AB98" s="8">
-        <f t="shared" ref="AB98:AB129" si="28">AA98+Y$2</f>
+        <f t="shared" ref="AB98:AB127" si="28">AA98+Y$2</f>
         <v>18.899999999999999</v>
       </c>
       <c r="AC98" s="8">
@@ -11069,7 +11069,7 @@
         <v>36.200000000000003</v>
       </c>
       <c r="AE98" s="8">
-        <f t="shared" ref="AE98:AE129" si="31">AD98+Y$2</f>
+        <f t="shared" ref="AE98:AE127" si="31">AD98+Y$2</f>
         <v>35.1</v>
       </c>
       <c r="AF98" s="8">
@@ -11081,7 +11081,7 @@
         <v>21.6</v>
       </c>
       <c r="AH98" s="8">
-        <f t="shared" ref="AH98:AH129" si="34">AG98+Y$2</f>
+        <f t="shared" ref="AH98:AH127" si="34">AG98+Y$2</f>
         <v>20.5</v>
       </c>
       <c r="AI98" s="10">
@@ -11089,7 +11089,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="99" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>1</v>
       </c>
@@ -11177,7 +11177,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="100" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A100">
         <v>1</v>
       </c>
@@ -11265,7 +11265,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="101" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A101">
         <v>1</v>
       </c>
@@ -11353,7 +11353,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="102" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A102">
         <v>1</v>
       </c>
@@ -11449,7 +11449,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="103" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A103">
         <v>1</v>
       </c>
@@ -11529,7 +11529,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="104" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A104">
         <v>1</v>
       </c>
@@ -11609,7 +11609,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="105" spans="1:35" ht="75" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:35" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A105">
         <v>1</v>
       </c>
@@ -11705,7 +11705,7 @@
         <v>67.2</v>
       </c>
     </row>
-    <row r="106" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A106">
         <v>1</v>
       </c>
@@ -11793,7 +11793,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="107" spans="1:35" ht="60" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A107">
         <v>1</v>
       </c>
@@ -11873,7 +11873,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="108" spans="1:35" ht="60" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A108">
         <v>1</v>
       </c>
@@ -11963,7 +11963,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="109" spans="1:35" ht="60" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A109">
         <v>1</v>
       </c>
@@ -12053,7 +12053,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="110" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A110">
         <v>1</v>
       </c>
@@ -12135,7 +12135,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="111" spans="1:35" ht="60" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:35" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A111">
         <v>1</v>
       </c>
@@ -12225,7 +12225,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="112" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A112">
         <v>1</v>
       </c>
@@ -12321,7 +12321,7 @@
         <v>71.599999999999994</v>
       </c>
     </row>
-    <row r="113" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A113">
         <v>1</v>
       </c>
@@ -12409,7 +12409,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="114" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A114">
         <v>1</v>
       </c>
@@ -12489,7 +12489,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="115" spans="1:35" ht="60" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A115">
         <v>1</v>
       </c>
@@ -12577,7 +12577,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="116" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A116">
         <v>1</v>
       </c>
@@ -12665,7 +12665,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="117" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A117">
         <v>1</v>
       </c>
@@ -12753,7 +12753,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="118" spans="1:35" ht="60" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:35" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A118">
         <v>1</v>
       </c>
@@ -12841,7 +12841,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="119" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A119">
         <v>1</v>
       </c>
@@ -12929,7 +12929,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="120" spans="1:35" ht="30" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A120">
         <v>1</v>
       </c>
@@ -13009,7 +13009,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="121" spans="1:35" ht="75" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:35" ht="72" x14ac:dyDescent="0.3">
       <c r="A121">
         <v>1</v>
       </c>
@@ -13089,7 +13089,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="122" spans="1:35" ht="75" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:35" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A122">
         <v>1</v>
       </c>
@@ -13185,7 +13185,7 @@
         <v>71.599999999999994</v>
       </c>
     </row>
-    <row r="123" spans="1:35" ht="75" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:35" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A123">
         <v>1</v>
       </c>
@@ -13273,7 +13273,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="124" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A124">
         <v>1</v>
       </c>
@@ -13369,7 +13369,7 @@
         <v>71.599999999999994</v>
       </c>
     </row>
-    <row r="125" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A125">
         <v>1</v>
       </c>
@@ -13459,7 +13459,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="126" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A126">
         <v>1</v>
       </c>
@@ -13547,7 +13547,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="127" spans="1:35" ht="45" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A127">
         <v>1</v>
       </c>
@@ -13627,7 +13627,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="128" spans="1:35" ht="60" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:35" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A128">
         <v>1</v>
       </c>
@@ -13715,40 +13715,40 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="129" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="129" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="O129"/>
     </row>
-    <row r="130" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="130" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="O130"/>
     </row>
-    <row r="131" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="131" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="O131"/>
     </row>
-    <row r="132" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="132" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="O132"/>
     </row>
-    <row r="133" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="133" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="O133"/>
     </row>
-    <row r="134" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="134" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="O134"/>
     </row>
-    <row r="135" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="135" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="O135"/>
     </row>
-    <row r="136" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="136" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="O136"/>
     </row>
-    <row r="137" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="137" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="O137"/>
     </row>
-    <row r="138" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="138" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="O138"/>
     </row>
-    <row r="139" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="139" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="O139"/>
     </row>
-    <row r="140" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="140" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B140" s="22"/>
       <c r="C140" s="22"/>
       <c r="D140" s="22"/>
@@ -13784,7 +13784,7 @@
       <c r="AH140" s="22"/>
       <c r="AI140" s="23"/>
     </row>
-    <row r="141" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="141" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B141" s="22"/>
       <c r="C141" s="22"/>
       <c r="D141" s="22"/>
@@ -13820,7 +13820,7 @@
       <c r="AH141" s="22"/>
       <c r="AI141" s="23"/>
     </row>
-    <row r="142" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="142" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B142" s="22"/>
       <c r="C142" s="22"/>
       <c r="D142" s="22"/>
@@ -13856,7 +13856,7 @@
       <c r="AH142" s="22"/>
       <c r="AI142" s="23"/>
     </row>
-    <row r="143" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="143" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B143" s="22"/>
       <c r="C143" s="22"/>
       <c r="D143" s="22"/>
@@ -13892,7 +13892,7 @@
       <c r="AH143" s="22"/>
       <c r="AI143" s="23"/>
     </row>
-    <row r="144" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="144" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B144" s="22"/>
       <c r="C144" s="22"/>
       <c r="D144" s="22"/>
@@ -13928,7 +13928,7 @@
       <c r="AH144" s="22"/>
       <c r="AI144" s="23"/>
     </row>
-    <row r="145" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="145" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B145" s="22"/>
       <c r="C145" s="22"/>
       <c r="D145" s="22"/>
@@ -13964,7 +13964,7 @@
       <c r="AH145" s="22"/>
       <c r="AI145" s="23"/>
     </row>
-    <row r="146" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="146" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B146" s="22"/>
       <c r="C146" s="22"/>
       <c r="D146" s="22"/>
@@ -14000,7 +14000,7 @@
       <c r="AH146" s="22"/>
       <c r="AI146" s="23"/>
     </row>
-    <row r="147" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="147" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B147" s="22"/>
       <c r="C147" s="22"/>
       <c r="D147" s="22"/>
@@ -14036,7 +14036,7 @@
       <c r="AH147" s="22"/>
       <c r="AI147" s="23"/>
     </row>
-    <row r="148" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="148" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B148" s="22"/>
       <c r="C148" s="22"/>
       <c r="D148" s="22"/>
@@ -14072,7 +14072,7 @@
       <c r="AH148" s="22"/>
       <c r="AI148" s="23"/>
     </row>
-    <row r="149" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="149" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B149" s="22"/>
       <c r="C149" s="22"/>
       <c r="D149" s="22"/>
@@ -14108,7 +14108,7 @@
       <c r="AH149" s="22"/>
       <c r="AI149" s="23"/>
     </row>
-    <row r="150" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="150" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B150" s="22"/>
       <c r="C150" s="22"/>
       <c r="D150" s="22"/>
@@ -14144,7 +14144,7 @@
       <c r="AH150" s="22"/>
       <c r="AI150" s="23"/>
     </row>
-    <row r="151" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="151" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B151" s="22"/>
       <c r="C151" s="22"/>
       <c r="D151" s="22"/>
@@ -14180,7 +14180,7 @@
       <c r="AH151" s="22"/>
       <c r="AI151" s="23"/>
     </row>
-    <row r="152" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="152" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B152" s="22"/>
       <c r="C152" s="22"/>
       <c r="D152" s="22"/>
@@ -14216,7 +14216,7 @@
       <c r="AH152" s="22"/>
       <c r="AI152" s="23"/>
     </row>
-    <row r="153" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="153" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B153" s="22"/>
       <c r="C153" s="22"/>
       <c r="D153" s="22"/>
@@ -14252,7 +14252,7 @@
       <c r="AH153" s="22"/>
       <c r="AI153" s="23"/>
     </row>
-    <row r="154" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="154" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B154" s="22"/>
       <c r="C154" s="22"/>
       <c r="D154" s="22"/>
@@ -14288,7 +14288,7 @@
       <c r="AH154" s="22"/>
       <c r="AI154" s="23"/>
     </row>
-    <row r="155" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="155" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B155" s="22"/>
       <c r="C155" s="22"/>
       <c r="D155" s="22"/>
@@ -14324,7 +14324,7 @@
       <c r="AH155" s="22"/>
       <c r="AI155" s="23"/>
     </row>
-    <row r="156" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="156" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B156" s="22"/>
       <c r="C156" s="22"/>
       <c r="D156" s="22"/>
@@ -14360,7 +14360,7 @@
       <c r="AH156" s="22"/>
       <c r="AI156" s="23"/>
     </row>
-    <row r="157" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="157" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B157" s="22"/>
       <c r="C157" s="22"/>
       <c r="D157" s="22"/>
@@ -14396,7 +14396,7 @@
       <c r="AH157" s="22"/>
       <c r="AI157" s="23"/>
     </row>
-    <row r="158" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="158" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B158" s="22"/>
       <c r="C158" s="22"/>
       <c r="D158" s="22"/>
@@ -14432,7 +14432,7 @@
       <c r="AH158" s="22"/>
       <c r="AI158" s="23"/>
     </row>
-    <row r="159" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="159" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B159" s="22"/>
       <c r="C159" s="22"/>
       <c r="D159" s="22"/>
@@ -14468,7 +14468,7 @@
       <c r="AH159" s="22"/>
       <c r="AI159" s="23"/>
     </row>
-    <row r="160" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="160" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B160" s="22"/>
       <c r="C160" s="22"/>
       <c r="D160" s="22"/>
@@ -14504,7 +14504,7 @@
       <c r="AH160" s="22"/>
       <c r="AI160" s="23"/>
     </row>
-    <row r="161" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="161" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B161" s="22"/>
       <c r="C161" s="22"/>
       <c r="D161" s="22"/>
@@ -14540,7 +14540,7 @@
       <c r="AH161" s="22"/>
       <c r="AI161" s="23"/>
     </row>
-    <row r="162" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="162" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B162" s="22"/>
       <c r="C162" s="22"/>
       <c r="D162" s="22"/>
@@ -14576,7 +14576,7 @@
       <c r="AH162" s="22"/>
       <c r="AI162" s="23"/>
     </row>
-    <row r="163" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="163" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B163" s="22"/>
       <c r="C163" s="22"/>
       <c r="D163" s="22"/>
@@ -14612,7 +14612,7 @@
       <c r="AH163" s="22"/>
       <c r="AI163" s="23"/>
     </row>
-    <row r="164" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="164" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B164" s="22"/>
       <c r="C164" s="22"/>
       <c r="D164" s="22"/>
@@ -14648,7 +14648,7 @@
       <c r="AH164" s="22"/>
       <c r="AI164" s="23"/>
     </row>
-    <row r="165" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="165" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B165" s="22"/>
       <c r="C165" s="22"/>
       <c r="D165" s="22"/>
@@ -14684,7 +14684,7 @@
       <c r="AH165" s="22"/>
       <c r="AI165" s="23"/>
     </row>
-    <row r="166" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="166" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B166" s="22"/>
       <c r="C166" s="22"/>
       <c r="D166" s="22"/>
@@ -14720,7 +14720,7 @@
       <c r="AH166" s="22"/>
       <c r="AI166" s="23"/>
     </row>
-    <row r="167" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="167" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B167" s="22"/>
       <c r="C167" s="22"/>
       <c r="D167" s="22"/>
@@ -14756,7 +14756,7 @@
       <c r="AH167" s="22"/>
       <c r="AI167" s="23"/>
     </row>
-    <row r="168" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="168" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B168" s="22"/>
       <c r="C168" s="22"/>
       <c r="D168" s="22"/>
@@ -14792,7 +14792,7 @@
       <c r="AH168" s="22"/>
       <c r="AI168" s="23"/>
     </row>
-    <row r="169" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="169" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B169" s="22"/>
       <c r="C169" s="22"/>
       <c r="D169" s="22"/>
@@ -14828,7 +14828,7 @@
       <c r="AH169" s="22"/>
       <c r="AI169" s="23"/>
     </row>
-    <row r="170" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="170" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B170" s="22"/>
       <c r="C170" s="22"/>
       <c r="D170" s="22"/>
@@ -14864,7 +14864,7 @@
       <c r="AH170" s="22"/>
       <c r="AI170" s="23"/>
     </row>
-    <row r="171" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="171" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B171" s="22"/>
       <c r="C171" s="22"/>
       <c r="D171" s="22"/>
@@ -14900,7 +14900,7 @@
       <c r="AH171" s="22"/>
       <c r="AI171" s="23"/>
     </row>
-    <row r="172" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="172" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B172" s="22"/>
       <c r="C172" s="22"/>
       <c r="D172" s="22"/>
@@ -14936,7 +14936,7 @@
       <c r="AH172" s="22"/>
       <c r="AI172" s="23"/>
     </row>
-    <row r="173" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="173" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B173" s="22"/>
       <c r="C173" s="22"/>
       <c r="D173" s="22"/>
@@ -14972,7 +14972,7 @@
       <c r="AH173" s="22"/>
       <c r="AI173" s="23"/>
     </row>
-    <row r="174" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="174" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B174" s="22"/>
       <c r="C174" s="22"/>
       <c r="D174" s="22"/>
@@ -15008,7 +15008,7 @@
       <c r="AH174" s="22"/>
       <c r="AI174" s="23"/>
     </row>
-    <row r="175" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="175" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B175" s="22"/>
       <c r="C175" s="22"/>
       <c r="D175" s="22"/>
@@ -15044,7 +15044,7 @@
       <c r="AH175" s="22"/>
       <c r="AI175" s="23"/>
     </row>
-    <row r="176" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="176" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B176" s="22"/>
       <c r="C176" s="22"/>
       <c r="D176" s="22"/>
@@ -15080,7 +15080,7 @@
       <c r="AH176" s="22"/>
       <c r="AI176" s="23"/>
     </row>
-    <row r="177" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="177" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B177" s="22"/>
       <c r="C177" s="22"/>
       <c r="D177" s="22"/>
@@ -15116,7 +15116,7 @@
       <c r="AH177" s="22"/>
       <c r="AI177" s="23"/>
     </row>
-    <row r="178" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="178" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B178" s="22"/>
       <c r="C178" s="22"/>
       <c r="D178" s="22"/>
@@ -15152,7 +15152,7 @@
       <c r="AH178" s="22"/>
       <c r="AI178" s="23"/>
     </row>
-    <row r="179" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="179" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B179" s="22"/>
       <c r="C179" s="22"/>
       <c r="D179" s="22"/>
@@ -15188,7 +15188,7 @@
       <c r="AH179" s="22"/>
       <c r="AI179" s="23"/>
     </row>
-    <row r="180" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="180" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B180" s="22"/>
       <c r="C180" s="22"/>
       <c r="D180" s="22"/>
@@ -15224,7 +15224,7 @@
       <c r="AH180" s="22"/>
       <c r="AI180" s="23"/>
     </row>
-    <row r="181" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="181" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B181" s="22"/>
       <c r="C181" s="22"/>
       <c r="D181" s="22"/>
@@ -15260,7 +15260,7 @@
       <c r="AH181" s="22"/>
       <c r="AI181" s="23"/>
     </row>
-    <row r="182" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="182" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B182" s="22"/>
       <c r="C182" s="22"/>
       <c r="D182" s="22"/>
@@ -15296,7 +15296,7 @@
       <c r="AH182" s="22"/>
       <c r="AI182" s="23"/>
     </row>
-    <row r="183" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="183" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B183" s="22"/>
       <c r="C183" s="22"/>
       <c r="D183" s="22"/>
@@ -15332,7 +15332,7 @@
       <c r="AH183" s="22"/>
       <c r="AI183" s="23"/>
     </row>
-    <row r="184" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="184" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B184" s="22"/>
       <c r="C184" s="22"/>
       <c r="D184" s="22"/>
@@ -15368,7 +15368,7 @@
       <c r="AH184" s="22"/>
       <c r="AI184" s="23"/>
     </row>
-    <row r="185" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="185" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B185" s="22"/>
       <c r="C185" s="22"/>
       <c r="D185" s="22"/>
@@ -15404,7 +15404,7 @@
       <c r="AH185" s="22"/>
       <c r="AI185" s="23"/>
     </row>
-    <row r="186" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="186" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B186" s="22"/>
       <c r="C186" s="22"/>
       <c r="D186" s="22"/>
@@ -15440,7 +15440,7 @@
       <c r="AH186" s="22"/>
       <c r="AI186" s="23"/>
     </row>
-    <row r="187" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="187" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B187" s="22"/>
       <c r="C187" s="22"/>
       <c r="D187" s="22"/>
@@ -15476,7 +15476,7 @@
       <c r="AH187" s="22"/>
       <c r="AI187" s="23"/>
     </row>
-    <row r="188" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="188" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B188" s="22"/>
       <c r="C188" s="22"/>
       <c r="D188" s="22"/>
@@ -15512,7 +15512,7 @@
       <c r="AH188" s="22"/>
       <c r="AI188" s="23"/>
     </row>
-    <row r="189" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="189" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B189" s="22"/>
       <c r="C189" s="22"/>
       <c r="D189" s="22"/>
@@ -15548,7 +15548,7 @@
       <c r="AH189" s="22"/>
       <c r="AI189" s="23"/>
     </row>
-    <row r="190" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="190" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B190" s="22"/>
       <c r="C190" s="22"/>
       <c r="D190" s="22"/>
@@ -15584,7 +15584,7 @@
       <c r="AH190" s="22"/>
       <c r="AI190" s="23"/>
     </row>
-    <row r="191" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="191" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B191" s="22"/>
       <c r="C191" s="22"/>
       <c r="D191" s="22"/>
@@ -15620,7 +15620,7 @@
       <c r="AH191" s="22"/>
       <c r="AI191" s="23"/>
     </row>
-    <row r="192" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="192" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B192" s="22"/>
       <c r="C192" s="22"/>
       <c r="D192" s="22"/>
@@ -15656,7 +15656,7 @@
       <c r="AH192" s="22"/>
       <c r="AI192" s="23"/>
     </row>
-    <row r="193" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="193" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B193" s="22"/>
       <c r="C193" s="22"/>
       <c r="D193" s="22"/>
@@ -15692,7 +15692,7 @@
       <c r="AH193" s="22"/>
       <c r="AI193" s="23"/>
     </row>
-    <row r="194" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="194" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B194" s="22"/>
       <c r="C194" s="22"/>
       <c r="D194" s="22"/>
@@ -15728,7 +15728,7 @@
       <c r="AH194" s="22"/>
       <c r="AI194" s="23"/>
     </row>
-    <row r="195" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="195" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B195" s="22"/>
       <c r="C195" s="22"/>
       <c r="D195" s="22"/>
@@ -15764,7 +15764,7 @@
       <c r="AH195" s="22"/>
       <c r="AI195" s="23"/>
     </row>
-    <row r="196" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="196" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B196" s="22"/>
       <c r="C196" s="22"/>
       <c r="D196" s="22"/>
@@ -15800,7 +15800,7 @@
       <c r="AH196" s="22"/>
       <c r="AI196" s="23"/>
     </row>
-    <row r="197" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="197" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B197" s="22"/>
       <c r="C197" s="22"/>
       <c r="D197" s="22"/>
@@ -15836,7 +15836,7 @@
       <c r="AH197" s="22"/>
       <c r="AI197" s="23"/>
     </row>
-    <row r="198" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="198" spans="2:35" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B198" s="22"/>
       <c r="C198" s="22"/>
       <c r="D198" s="22"/>
@@ -15872,13 +15872,13 @@
       <c r="AH198" s="22"/>
       <c r="AI198" s="23"/>
     </row>
-    <row r="199" spans="2:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="199" spans="2:35" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C199" s="22"/>
     </row>
-    <row r="200" spans="2:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="200" spans="2:35" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C200" s="22"/>
     </row>
-    <row r="201" spans="2:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="201" spans="2:35" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C201" s="22"/>
     </row>
   </sheetData>

</xml_diff>